<commit_message>
Upload LF_Ball_Mill_Metallurgical_Report.xlsx via Zeta Client · 62 sel berubah · Data Sampel, Tren Harian
</commit_message>
<xml_diff>
--- a/PRODUKSI/REPORT/LF_Ball_Mill_Metallurgical_Report.xlsx
+++ b/PRODUKSI/REPORT/LF_Ball_Mill_Metallurgical_Report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ramda\Documents\Zeta_Edit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80C2D6AE-724D-46C9-BF2C-285A81FAAB13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{496E57BD-7A55-4A4F-B224-1C3F11CAC065}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="54">
   <si>
     <t>Periode</t>
   </si>
@@ -221,23 +221,13 @@
   <si>
     <t xml:space="preserve">Leach Feed BALL MILL </t>
   </si>
-  <si>
-    <t>Max</t>
-  </si>
-  <si>
-    <t>Min</t>
-  </si>
-  <si>
-    <t>Average</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\ mmm\ yyyy"/>
-    <numFmt numFmtId="170" formatCode="0.000"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -262,7 +252,7 @@
       <name val="Carlito"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -286,8 +276,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -295,11 +291,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -326,14 +337,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3421,7 +3443,7 @@
       </c>
     </row>
     <row r="21" spans="2:23">
-      <c r="W21" s="17"/>
+      <c r="W21" s="14"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3431,7 +3453,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
@@ -4450,6 +4472,23 @@
       </c>
       <c r="H39">
         <v>11.662100000000001</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
+      <c r="A40" s="2">
+        <v>46312</v>
+      </c>
+      <c r="B40">
+        <v>8</v>
+      </c>
+      <c r="C40">
+        <v>0.71199999999999997</v>
+      </c>
+      <c r="D40">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="E40">
+        <v>8.41</v>
       </c>
     </row>
   </sheetData>
@@ -4613,7 +4652,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:I231"/>
+  <dimension ref="A1:I236"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -4654,7 +4693,7 @@
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="14">
+      <c r="B2" s="16">
         <v>1</v>
       </c>
       <c r="C2" s="5" t="s">
@@ -4680,7 +4719,7 @@
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="14"/>
+      <c r="B3" s="16"/>
       <c r="C3" s="5" t="s">
         <v>37</v>
       </c>
@@ -4704,7 +4743,7 @@
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" s="14"/>
+      <c r="B4" s="16"/>
       <c r="C4" s="5" t="s">
         <v>38</v>
       </c>
@@ -4728,7 +4767,7 @@
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" s="14"/>
+      <c r="B5" s="16"/>
       <c r="C5" s="5" t="s">
         <v>39</v>
       </c>
@@ -4752,7 +4791,7 @@
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" s="14"/>
+      <c r="B6" s="16"/>
       <c r="C6" s="5" t="s">
         <v>40</v>
       </c>
@@ -4776,7 +4815,7 @@
       <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7" s="14"/>
+      <c r="B7" s="16"/>
       <c r="C7" s="5" t="s">
         <v>41</v>
       </c>
@@ -4800,7 +4839,7 @@
       <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8" s="14"/>
+      <c r="B8" s="16"/>
       <c r="C8" s="5" t="s">
         <v>36</v>
       </c>
@@ -4824,7 +4863,7 @@
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" s="14"/>
+      <c r="B9" s="16"/>
       <c r="C9" s="5" t="s">
         <v>37</v>
       </c>
@@ -4848,7 +4887,7 @@
       <c r="A10">
         <v>9</v>
       </c>
-      <c r="B10" s="14"/>
+      <c r="B10" s="16"/>
       <c r="C10" s="5" t="s">
         <v>38</v>
       </c>
@@ -4872,7 +4911,7 @@
       <c r="A11">
         <v>10</v>
       </c>
-      <c r="B11" s="14"/>
+      <c r="B11" s="16"/>
       <c r="C11" s="5" t="s">
         <v>39</v>
       </c>
@@ -4896,7 +4935,7 @@
       <c r="A12">
         <v>11</v>
       </c>
-      <c r="B12" s="14"/>
+      <c r="B12" s="16"/>
       <c r="C12" s="5" t="s">
         <v>40</v>
       </c>
@@ -4920,7 +4959,7 @@
       <c r="A13">
         <v>12</v>
       </c>
-      <c r="B13" s="14"/>
+      <c r="B13" s="16"/>
       <c r="C13" s="5" t="s">
         <v>41</v>
       </c>
@@ -5162,7 +5201,7 @@
       <c r="A23">
         <v>22</v>
       </c>
-      <c r="B23" s="14">
+      <c r="B23" s="16">
         <v>3</v>
       </c>
       <c r="C23" s="5" t="s">
@@ -5188,7 +5227,7 @@
       <c r="A24">
         <v>23</v>
       </c>
-      <c r="B24" s="14"/>
+      <c r="B24" s="16"/>
       <c r="C24" s="5" t="s">
         <v>40</v>
       </c>
@@ -5212,7 +5251,7 @@
       <c r="A25">
         <v>24</v>
       </c>
-      <c r="B25" s="14"/>
+      <c r="B25" s="16"/>
       <c r="C25" s="5" t="s">
         <v>41</v>
       </c>
@@ -5236,7 +5275,7 @@
       <c r="A26">
         <v>25</v>
       </c>
-      <c r="B26" s="14"/>
+      <c r="B26" s="16"/>
       <c r="C26" s="5" t="s">
         <v>36</v>
       </c>
@@ -5260,7 +5299,7 @@
       <c r="A27">
         <v>26</v>
       </c>
-      <c r="B27" s="14"/>
+      <c r="B27" s="16"/>
       <c r="C27" s="5" t="s">
         <v>37</v>
       </c>
@@ -5284,7 +5323,7 @@
       <c r="A28">
         <v>27</v>
       </c>
-      <c r="B28" s="14"/>
+      <c r="B28" s="16"/>
       <c r="C28" s="5" t="s">
         <v>38</v>
       </c>
@@ -5308,7 +5347,7 @@
       <c r="A29">
         <v>28</v>
       </c>
-      <c r="B29" s="14"/>
+      <c r="B29" s="16"/>
       <c r="C29" s="5" t="s">
         <v>39</v>
       </c>
@@ -5332,7 +5371,7 @@
       <c r="A30">
         <v>29</v>
       </c>
-      <c r="B30" s="14"/>
+      <c r="B30" s="16"/>
       <c r="C30" s="5" t="s">
         <v>40</v>
       </c>
@@ -5356,7 +5395,7 @@
       <c r="A31">
         <v>30</v>
       </c>
-      <c r="B31" s="14"/>
+      <c r="B31" s="16"/>
       <c r="C31" s="5" t="s">
         <v>41</v>
       </c>
@@ -5380,7 +5419,7 @@
       <c r="A32">
         <v>31</v>
       </c>
-      <c r="B32" s="14"/>
+      <c r="B32" s="16"/>
       <c r="C32" s="5" t="s">
         <v>36</v>
       </c>
@@ -5404,7 +5443,7 @@
       <c r="A33">
         <v>32</v>
       </c>
-      <c r="B33" s="14"/>
+      <c r="B33" s="16"/>
       <c r="C33" s="5" t="s">
         <v>37</v>
       </c>
@@ -5428,7 +5467,7 @@
       <c r="A34">
         <v>33</v>
       </c>
-      <c r="B34" s="14"/>
+      <c r="B34" s="16"/>
       <c r="C34" s="5" t="s">
         <v>38</v>
       </c>
@@ -5796,7 +5835,7 @@
       <c r="A50">
         <v>49</v>
       </c>
-      <c r="B50" s="14">
+      <c r="B50" s="16">
         <v>5</v>
       </c>
       <c r="C50" s="5" t="s">
@@ -5822,7 +5861,7 @@
       <c r="A51">
         <v>50</v>
       </c>
-      <c r="B51" s="14"/>
+      <c r="B51" s="16"/>
       <c r="C51" s="5" t="s">
         <v>37</v>
       </c>
@@ -5846,7 +5885,7 @@
       <c r="A52">
         <v>51</v>
       </c>
-      <c r="B52" s="14"/>
+      <c r="B52" s="16"/>
       <c r="C52" s="5" t="s">
         <v>38</v>
       </c>
@@ -5870,7 +5909,7 @@
       <c r="A53">
         <v>52</v>
       </c>
-      <c r="B53" s="14"/>
+      <c r="B53" s="16"/>
       <c r="C53" s="5" t="s">
         <v>39</v>
       </c>
@@ -5894,7 +5933,7 @@
       <c r="A54">
         <v>53</v>
       </c>
-      <c r="B54" s="14"/>
+      <c r="B54" s="16"/>
       <c r="C54" s="5" t="s">
         <v>40</v>
       </c>
@@ -5918,7 +5957,7 @@
       <c r="A55">
         <v>54</v>
       </c>
-      <c r="B55" s="14"/>
+      <c r="B55" s="16"/>
       <c r="C55" s="5" t="s">
         <v>41</v>
       </c>
@@ -5942,7 +5981,7 @@
       <c r="A56">
         <v>55</v>
       </c>
-      <c r="B56" s="14"/>
+      <c r="B56" s="16"/>
       <c r="C56" s="5" t="s">
         <v>36</v>
       </c>
@@ -5966,7 +6005,7 @@
       <c r="A57">
         <v>56</v>
       </c>
-      <c r="B57" s="14"/>
+      <c r="B57" s="16"/>
       <c r="C57" s="5" t="s">
         <v>37</v>
       </c>
@@ -5990,7 +6029,7 @@
       <c r="A58">
         <v>57</v>
       </c>
-      <c r="B58" s="14"/>
+      <c r="B58" s="16"/>
       <c r="C58" s="5" t="s">
         <v>38</v>
       </c>
@@ -6160,7 +6199,7 @@
       <c r="A65">
         <v>64</v>
       </c>
-      <c r="B65" s="14">
+      <c r="B65" s="16">
         <v>7</v>
       </c>
       <c r="C65" s="5" t="s">
@@ -6186,7 +6225,7 @@
       <c r="A66">
         <v>65</v>
       </c>
-      <c r="B66" s="14"/>
+      <c r="B66" s="16"/>
       <c r="C66" s="5" t="s">
         <v>40</v>
       </c>
@@ -6210,7 +6249,7 @@
       <c r="A67">
         <v>66</v>
       </c>
-      <c r="B67" s="14"/>
+      <c r="B67" s="16"/>
       <c r="C67" s="5" t="s">
         <v>41</v>
       </c>
@@ -6234,7 +6273,7 @@
       <c r="A68">
         <v>67</v>
       </c>
-      <c r="B68" s="14"/>
+      <c r="B68" s="16"/>
       <c r="C68" s="5" t="s">
         <v>36</v>
       </c>
@@ -6258,7 +6297,7 @@
       <c r="A69">
         <v>68</v>
       </c>
-      <c r="B69" s="14"/>
+      <c r="B69" s="16"/>
       <c r="C69" s="5" t="s">
         <v>37</v>
       </c>
@@ -6282,7 +6321,7 @@
       <c r="A70">
         <v>69</v>
       </c>
-      <c r="B70" s="14"/>
+      <c r="B70" s="16"/>
       <c r="C70" s="5" t="s">
         <v>38</v>
       </c>
@@ -6306,7 +6345,7 @@
       <c r="A71">
         <v>70</v>
       </c>
-      <c r="B71" s="14"/>
+      <c r="B71" s="16"/>
       <c r="C71" s="5" t="s">
         <v>39</v>
       </c>
@@ -6330,7 +6369,7 @@
       <c r="A72">
         <v>71</v>
       </c>
-      <c r="B72" s="14"/>
+      <c r="B72" s="16"/>
       <c r="C72" s="5" t="s">
         <v>40</v>
       </c>
@@ -6354,7 +6393,7 @@
       <c r="A73">
         <v>72</v>
       </c>
-      <c r="B73" s="14"/>
+      <c r="B73" s="16"/>
       <c r="C73" s="5" t="s">
         <v>41</v>
       </c>
@@ -6668,7 +6707,7 @@
       <c r="A86">
         <v>85</v>
       </c>
-      <c r="B86" s="14">
+      <c r="B86" s="16">
         <v>9</v>
       </c>
       <c r="C86" s="5" t="s">
@@ -6694,7 +6733,7 @@
       <c r="A87">
         <v>86</v>
       </c>
-      <c r="B87" s="14"/>
+      <c r="B87" s="16"/>
       <c r="C87" s="5" t="s">
         <v>37</v>
       </c>
@@ -6718,7 +6757,7 @@
       <c r="A88">
         <v>87</v>
       </c>
-      <c r="B88" s="14"/>
+      <c r="B88" s="16"/>
       <c r="C88" s="5" t="s">
         <v>38</v>
       </c>
@@ -6742,7 +6781,7 @@
       <c r="A89">
         <v>88</v>
       </c>
-      <c r="B89" s="14"/>
+      <c r="B89" s="16"/>
       <c r="C89" s="5" t="s">
         <v>39</v>
       </c>
@@ -6766,7 +6805,7 @@
       <c r="A90">
         <v>89</v>
       </c>
-      <c r="B90" s="14"/>
+      <c r="B90" s="16"/>
       <c r="C90" s="5" t="s">
         <v>40</v>
       </c>
@@ -6790,7 +6829,7 @@
       <c r="A91">
         <v>90</v>
       </c>
-      <c r="B91" s="14"/>
+      <c r="B91" s="16"/>
       <c r="C91" s="5" t="s">
         <v>41</v>
       </c>
@@ -6814,7 +6853,7 @@
       <c r="A92">
         <v>91</v>
       </c>
-      <c r="B92" s="14"/>
+      <c r="B92" s="16"/>
       <c r="C92" s="5" t="s">
         <v>36</v>
       </c>
@@ -6838,7 +6877,7 @@
       <c r="A93">
         <v>92</v>
       </c>
-      <c r="B93" s="14"/>
+      <c r="B93" s="16"/>
       <c r="C93" s="5" t="s">
         <v>37</v>
       </c>
@@ -6862,7 +6901,7 @@
       <c r="A94">
         <v>93</v>
       </c>
-      <c r="B94" s="14"/>
+      <c r="B94" s="16"/>
       <c r="C94" s="5" t="s">
         <v>38</v>
       </c>
@@ -6886,7 +6925,7 @@
       <c r="A95">
         <v>94</v>
       </c>
-      <c r="B95" s="14"/>
+      <c r="B95" s="16"/>
       <c r="C95" s="5" t="s">
         <v>39</v>
       </c>
@@ -6910,7 +6949,7 @@
       <c r="A96">
         <v>95</v>
       </c>
-      <c r="B96" s="14"/>
+      <c r="B96" s="16"/>
       <c r="C96" s="5" t="s">
         <v>40</v>
       </c>
@@ -6934,7 +6973,7 @@
       <c r="A97">
         <v>96</v>
       </c>
-      <c r="B97" s="14"/>
+      <c r="B97" s="16"/>
       <c r="C97" s="5" t="s">
         <v>41</v>
       </c>
@@ -7464,7 +7503,7 @@
       <c r="A119">
         <v>118</v>
       </c>
-      <c r="B119" s="14">
+      <c r="B119" s="16">
         <v>11</v>
       </c>
       <c r="C119" s="5" t="s">
@@ -7490,7 +7529,7 @@
       <c r="A120">
         <v>119</v>
       </c>
-      <c r="B120" s="14"/>
+      <c r="B120" s="16"/>
       <c r="C120" s="5" t="s">
         <v>40</v>
       </c>
@@ -7514,7 +7553,7 @@
       <c r="A121">
         <v>120</v>
       </c>
-      <c r="B121" s="14"/>
+      <c r="B121" s="16"/>
       <c r="C121" s="5" t="s">
         <v>41</v>
       </c>
@@ -7538,7 +7577,7 @@
       <c r="A122">
         <v>121</v>
       </c>
-      <c r="B122" s="14"/>
+      <c r="B122" s="16"/>
       <c r="C122" s="5" t="s">
         <v>36</v>
       </c>
@@ -7562,7 +7601,7 @@
       <c r="A123">
         <v>122</v>
       </c>
-      <c r="B123" s="14"/>
+      <c r="B123" s="16"/>
       <c r="C123" s="5" t="s">
         <v>37</v>
       </c>
@@ -7586,7 +7625,7 @@
       <c r="A124">
         <v>123</v>
       </c>
-      <c r="B124" s="14"/>
+      <c r="B124" s="16"/>
       <c r="C124" s="5" t="s">
         <v>38</v>
       </c>
@@ -7610,7 +7649,7 @@
       <c r="A125">
         <v>124</v>
       </c>
-      <c r="B125" s="14"/>
+      <c r="B125" s="16"/>
       <c r="C125" s="5" t="s">
         <v>39</v>
       </c>
@@ -7628,7 +7667,7 @@
       <c r="A126">
         <v>125</v>
       </c>
-      <c r="B126" s="14"/>
+      <c r="B126" s="16"/>
       <c r="C126" s="5" t="s">
         <v>40</v>
       </c>
@@ -7646,7 +7685,7 @@
       <c r="A127">
         <v>126</v>
       </c>
-      <c r="B127" s="14"/>
+      <c r="B127" s="16"/>
       <c r="C127" s="5" t="s">
         <v>41</v>
       </c>
@@ -8098,7 +8137,7 @@
       <c r="A146">
         <v>145</v>
       </c>
-      <c r="B146" s="14">
+      <c r="B146" s="16">
         <v>13</v>
       </c>
       <c r="C146" s="5" t="s">
@@ -8124,7 +8163,7 @@
       <c r="A147">
         <v>146</v>
       </c>
-      <c r="B147" s="14"/>
+      <c r="B147" s="16"/>
       <c r="C147" s="5" t="s">
         <v>40</v>
       </c>
@@ -8148,7 +8187,7 @@
       <c r="A148">
         <v>147</v>
       </c>
-      <c r="B148" s="14"/>
+      <c r="B148" s="16"/>
       <c r="C148" s="5" t="s">
         <v>41</v>
       </c>
@@ -8172,7 +8211,7 @@
       <c r="A149">
         <v>148</v>
       </c>
-      <c r="B149" s="14"/>
+      <c r="B149" s="16"/>
       <c r="C149" s="5" t="s">
         <v>36</v>
       </c>
@@ -8196,7 +8235,7 @@
       <c r="A150">
         <v>149</v>
       </c>
-      <c r="B150" s="14"/>
+      <c r="B150" s="16"/>
       <c r="C150" s="5" t="s">
         <v>37</v>
       </c>
@@ -8220,7 +8259,7 @@
       <c r="A151">
         <v>150</v>
       </c>
-      <c r="B151" s="14"/>
+      <c r="B151" s="16"/>
       <c r="C151" s="5" t="s">
         <v>38</v>
       </c>
@@ -8244,7 +8283,7 @@
       <c r="A152">
         <v>151</v>
       </c>
-      <c r="B152" s="14"/>
+      <c r="B152" s="16"/>
       <c r="C152" s="5" t="s">
         <v>39</v>
       </c>
@@ -8268,7 +8307,7 @@
       <c r="A153">
         <v>152</v>
       </c>
-      <c r="B153" s="14"/>
+      <c r="B153" s="16"/>
       <c r="C153" s="5" t="s">
         <v>40</v>
       </c>
@@ -8292,7 +8331,7 @@
       <c r="A154">
         <v>153</v>
       </c>
-      <c r="B154" s="14"/>
+      <c r="B154" s="16"/>
       <c r="C154" s="5" t="s">
         <v>41</v>
       </c>
@@ -8316,7 +8355,7 @@
       <c r="A155">
         <v>154</v>
       </c>
-      <c r="B155" s="14"/>
+      <c r="B155" s="16"/>
       <c r="C155" s="5" t="s">
         <v>36</v>
       </c>
@@ -8344,7 +8383,7 @@
       <c r="A156">
         <v>155</v>
       </c>
-      <c r="B156" s="14"/>
+      <c r="B156" s="16"/>
       <c r="C156" s="5" t="s">
         <v>37</v>
       </c>
@@ -8368,7 +8407,7 @@
       <c r="A157">
         <v>156</v>
       </c>
-      <c r="B157" s="14"/>
+      <c r="B157" s="16"/>
       <c r="C157" s="5" t="s">
         <v>38</v>
       </c>
@@ -8392,7 +8431,7 @@
       <c r="A158">
         <v>157</v>
       </c>
-      <c r="B158" s="14"/>
+      <c r="B158" s="16"/>
       <c r="C158" s="5" t="s">
         <v>39</v>
       </c>
@@ -8416,7 +8455,7 @@
       <c r="A159">
         <v>158</v>
       </c>
-      <c r="B159" s="14"/>
+      <c r="B159" s="16"/>
       <c r="C159" s="5" t="s">
         <v>40</v>
       </c>
@@ -8440,7 +8479,7 @@
       <c r="A160">
         <v>159</v>
       </c>
-      <c r="B160" s="14"/>
+      <c r="B160" s="16"/>
       <c r="C160" s="5" t="s">
         <v>41</v>
       </c>
@@ -8682,7 +8721,7 @@
       <c r="A170">
         <v>169</v>
       </c>
-      <c r="B170" s="14">
+      <c r="B170" s="16">
         <v>15</v>
       </c>
       <c r="C170" s="5" t="s">
@@ -8708,7 +8747,7 @@
       <c r="A171">
         <v>170</v>
       </c>
-      <c r="B171" s="14"/>
+      <c r="B171" s="16"/>
       <c r="C171" s="5" t="s">
         <v>40</v>
       </c>
@@ -8732,7 +8771,7 @@
       <c r="A172">
         <v>171</v>
       </c>
-      <c r="B172" s="14"/>
+      <c r="B172" s="16"/>
       <c r="C172" s="5" t="s">
         <v>41</v>
       </c>
@@ -8756,7 +8795,7 @@
       <c r="A173">
         <v>172</v>
       </c>
-      <c r="B173" s="14"/>
+      <c r="B173" s="16"/>
       <c r="C173" s="5" t="s">
         <v>36</v>
       </c>
@@ -8780,7 +8819,7 @@
       <c r="A174">
         <v>173</v>
       </c>
-      <c r="B174" s="14"/>
+      <c r="B174" s="16"/>
       <c r="C174" s="5" t="s">
         <v>37</v>
       </c>
@@ -8804,7 +8843,7 @@
       <c r="A175">
         <v>174</v>
       </c>
-      <c r="B175" s="14"/>
+      <c r="B175" s="16"/>
       <c r="C175" s="5" t="s">
         <v>38</v>
       </c>
@@ -8822,7 +8861,7 @@
       <c r="A176">
         <v>175</v>
       </c>
-      <c r="B176" s="14"/>
+      <c r="B176" s="16"/>
       <c r="C176" s="5" t="s">
         <v>39</v>
       </c>
@@ -8840,7 +8879,7 @@
       <c r="A177">
         <v>176</v>
       </c>
-      <c r="B177" s="14"/>
+      <c r="B177" s="16"/>
       <c r="C177" s="5" t="s">
         <v>40</v>
       </c>
@@ -8858,7 +8897,7 @@
       <c r="A178">
         <v>177</v>
       </c>
-      <c r="B178" s="14"/>
+      <c r="B178" s="16"/>
       <c r="C178" s="5" t="s">
         <v>41</v>
       </c>
@@ -9166,7 +9205,7 @@
       <c r="A191">
         <v>190</v>
       </c>
-      <c r="B191" s="14">
+      <c r="B191" s="16">
         <v>17</v>
       </c>
       <c r="C191" s="5" t="s">
@@ -9192,7 +9231,7 @@
       <c r="A192">
         <v>191</v>
       </c>
-      <c r="B192" s="14"/>
+      <c r="B192" s="16"/>
       <c r="C192" s="5" t="s">
         <v>37</v>
       </c>
@@ -9216,7 +9255,7 @@
       <c r="A193">
         <v>192</v>
       </c>
-      <c r="B193" s="14"/>
+      <c r="B193" s="16"/>
       <c r="C193" s="5" t="s">
         <v>38</v>
       </c>
@@ -9240,7 +9279,7 @@
       <c r="A194">
         <v>193</v>
       </c>
-      <c r="B194" s="14"/>
+      <c r="B194" s="16"/>
       <c r="C194" s="5" t="s">
         <v>39</v>
       </c>
@@ -9264,7 +9303,7 @@
       <c r="A195">
         <v>194</v>
       </c>
-      <c r="B195" s="14"/>
+      <c r="B195" s="16"/>
       <c r="C195" s="5" t="s">
         <v>40</v>
       </c>
@@ -9288,7 +9327,7 @@
       <c r="A196">
         <v>195</v>
       </c>
-      <c r="B196" s="14"/>
+      <c r="B196" s="16"/>
       <c r="C196" s="5" t="s">
         <v>41</v>
       </c>
@@ -9312,7 +9351,7 @@
       <c r="A197">
         <v>196</v>
       </c>
-      <c r="B197" s="14"/>
+      <c r="B197" s="16"/>
       <c r="C197" s="5" t="s">
         <v>36</v>
       </c>
@@ -9336,7 +9375,7 @@
       <c r="A198">
         <v>197</v>
       </c>
-      <c r="B198" s="14"/>
+      <c r="B198" s="16"/>
       <c r="C198" s="5" t="s">
         <v>37</v>
       </c>
@@ -9360,7 +9399,7 @@
       <c r="A199">
         <v>198</v>
       </c>
-      <c r="B199" s="14"/>
+      <c r="B199" s="16"/>
       <c r="C199" s="5" t="s">
         <v>38</v>
       </c>
@@ -9602,7 +9641,7 @@
       <c r="A209">
         <v>208</v>
       </c>
-      <c r="B209" s="14">
+      <c r="B209" s="16">
         <v>19</v>
       </c>
       <c r="C209" s="5" t="s">
@@ -9622,7 +9661,7 @@
       <c r="A210">
         <v>209</v>
       </c>
-      <c r="B210" s="14"/>
+      <c r="B210" s="16"/>
       <c r="C210" s="5" t="s">
         <v>37</v>
       </c>
@@ -9640,7 +9679,7 @@
       <c r="A211">
         <v>210</v>
       </c>
-      <c r="B211" s="14"/>
+      <c r="B211" s="16"/>
       <c r="C211" s="5" t="s">
         <v>38</v>
       </c>
@@ -9658,7 +9697,7 @@
       <c r="A212">
         <v>211</v>
       </c>
-      <c r="B212" s="14"/>
+      <c r="B212" s="16"/>
       <c r="C212" s="5" t="s">
         <v>39</v>
       </c>
@@ -9682,7 +9721,7 @@
       <c r="A213">
         <v>212</v>
       </c>
-      <c r="B213" s="14"/>
+      <c r="B213" s="16"/>
       <c r="C213" s="5" t="s">
         <v>40</v>
       </c>
@@ -9706,7 +9745,7 @@
       <c r="A214">
         <v>213</v>
       </c>
-      <c r="B214" s="14"/>
+      <c r="B214" s="16"/>
       <c r="C214" s="5" t="s">
         <v>41</v>
       </c>
@@ -9730,7 +9769,7 @@
       <c r="A215">
         <v>214</v>
       </c>
-      <c r="B215" s="14"/>
+      <c r="B215" s="16"/>
       <c r="C215" s="5" t="s">
         <v>42</v>
       </c>
@@ -9754,7 +9793,7 @@
       <c r="A216">
         <v>215</v>
       </c>
-      <c r="B216" s="14"/>
+      <c r="B216" s="16"/>
       <c r="C216" s="5" t="s">
         <v>43</v>
       </c>
@@ -9778,7 +9817,7 @@
       <c r="A217">
         <v>216</v>
       </c>
-      <c r="B217" s="14"/>
+      <c r="B217" s="16"/>
       <c r="C217" s="5" t="s">
         <v>44</v>
       </c>
@@ -9802,7 +9841,7 @@
       <c r="A218">
         <v>217</v>
       </c>
-      <c r="B218" s="14"/>
+      <c r="B218" s="16"/>
       <c r="C218" s="5" t="s">
         <v>45</v>
       </c>
@@ -9826,7 +9865,7 @@
       <c r="A219">
         <v>218</v>
       </c>
-      <c r="B219" s="14"/>
+      <c r="B219" s="16"/>
       <c r="C219" s="5" t="s">
         <v>46</v>
       </c>
@@ -9850,7 +9889,7 @@
       <c r="A220">
         <v>219</v>
       </c>
-      <c r="B220" s="14"/>
+      <c r="B220" s="16"/>
       <c r="C220" s="5" t="s">
         <v>47</v>
       </c>
@@ -9874,7 +9913,7 @@
       <c r="A221">
         <v>220</v>
       </c>
-      <c r="B221" s="14"/>
+      <c r="B221" s="16"/>
       <c r="C221" s="5" t="s">
         <v>48</v>
       </c>
@@ -9898,7 +9937,7 @@
       <c r="A222">
         <v>221</v>
       </c>
-      <c r="B222" s="14"/>
+      <c r="B222" s="16"/>
       <c r="C222" s="5" t="s">
         <v>36</v>
       </c>
@@ -9922,7 +9961,7 @@
       <c r="A223">
         <v>222</v>
       </c>
-      <c r="B223" s="14"/>
+      <c r="B223" s="16"/>
       <c r="C223" s="5" t="s">
         <v>37</v>
       </c>
@@ -9946,7 +9985,7 @@
       <c r="A224">
         <v>223</v>
       </c>
-      <c r="B224" s="14"/>
+      <c r="B224" s="16"/>
       <c r="C224" s="5" t="s">
         <v>38</v>
       </c>
@@ -9970,7 +10009,7 @@
       <c r="A225">
         <v>224</v>
       </c>
-      <c r="B225" s="14"/>
+      <c r="B225" s="16"/>
       <c r="C225" s="5" t="s">
         <v>49</v>
       </c>
@@ -9994,7 +10033,7 @@
       <c r="A226">
         <v>225</v>
       </c>
-      <c r="B226" s="14"/>
+      <c r="B226" s="16"/>
       <c r="C226" s="5" t="s">
         <v>50</v>
       </c>
@@ -10018,7 +10057,7 @@
       <c r="A227">
         <v>226</v>
       </c>
-      <c r="B227" s="14"/>
+      <c r="B227" s="16"/>
       <c r="C227" s="5" t="s">
         <v>51</v>
       </c>
@@ -10042,7 +10081,7 @@
       <c r="A228">
         <v>227</v>
       </c>
-      <c r="B228" s="14"/>
+      <c r="B228" s="16"/>
       <c r="C228" s="5" t="s">
         <v>52</v>
       </c>
@@ -10063,58 +10102,209 @@
       </c>
     </row>
     <row r="229" spans="1:8">
-      <c r="D229" t="s">
-        <v>54</v>
-      </c>
-      <c r="E229">
-        <f>MAX(E2:E228)</f>
-        <v>1.468</v>
-      </c>
-      <c r="F229">
-        <f t="shared" ref="F229:G229" si="0">MAX(F2:F228)</f>
-        <v>10.11</v>
-      </c>
-      <c r="G229">
-        <f t="shared" si="0"/>
-        <v>27.939</v>
+      <c r="A229">
+        <v>228</v>
+      </c>
+      <c r="B229" s="18">
+        <v>20</v>
+      </c>
+      <c r="C229" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="D229" s="17">
+        <v>46312</v>
+      </c>
+      <c r="E229" s="19">
+        <v>0.63200000000000001</v>
+      </c>
+      <c r="F229" s="19">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="G229" s="19">
+        <v>8.07</v>
+      </c>
+      <c r="H229" s="20" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="230" spans="1:8">
-      <c r="D230" t="s">
-        <v>55</v>
-      </c>
-      <c r="E230">
-        <f>MIN(E2:E228)</f>
-        <v>0.219</v>
-      </c>
-      <c r="F230">
-        <f t="shared" ref="F230:G230" si="1">MIN(F2:F228)</f>
-        <v>0.01</v>
-      </c>
-      <c r="G230">
-        <f t="shared" si="1"/>
-        <v>5.9560000000000004</v>
+      <c r="A230">
+        <v>229</v>
+      </c>
+      <c r="B230" s="18"/>
+      <c r="C230" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="D230" s="17">
+        <v>46312</v>
+      </c>
+      <c r="E230" s="19">
+        <v>0.68600000000000005</v>
+      </c>
+      <c r="F230" s="19">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="G230" s="19">
+        <v>8.31</v>
+      </c>
+      <c r="H230" s="20" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="231" spans="1:8">
-      <c r="D231" t="s">
-        <v>56</v>
-      </c>
-      <c r="E231" s="16">
-        <f>AVERAGE(E2:E228)</f>
-        <v>0.58585046728971923</v>
-      </c>
-      <c r="F231" s="16">
-        <f t="shared" ref="F231:G231" si="2">AVERAGE(F2:F228)</f>
-        <v>0.83742056074766358</v>
-      </c>
-      <c r="G231" s="16">
-        <f t="shared" si="2"/>
-        <v>12.438074766355133</v>
+      <c r="A231">
+        <v>230</v>
+      </c>
+      <c r="B231" s="18"/>
+      <c r="C231" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="D231" s="17">
+        <v>46312</v>
+      </c>
+      <c r="E231" s="19">
+        <v>0.69</v>
+      </c>
+      <c r="F231" s="19">
+        <v>0.52</v>
+      </c>
+      <c r="G231" s="19">
+        <v>8.7899999999999991</v>
+      </c>
+      <c r="H231" s="20" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="232" spans="1:8">
+      <c r="A232">
+        <v>231</v>
+      </c>
+      <c r="B232" s="18"/>
+      <c r="C232" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="D232" s="17">
+        <v>46312</v>
+      </c>
+      <c r="E232" s="19">
+        <v>0.75900000000000001</v>
+      </c>
+      <c r="F232" s="19">
+        <v>0.53</v>
+      </c>
+      <c r="G232" s="19">
+        <v>8.43</v>
+      </c>
+      <c r="H232" s="20" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="233" spans="1:8">
+      <c r="A233">
+        <v>232</v>
+      </c>
+      <c r="B233" s="18"/>
+      <c r="C233" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="D233" s="17">
+        <v>46312</v>
+      </c>
+      <c r="E233" s="19">
+        <v>0.746</v>
+      </c>
+      <c r="F233" s="19">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G233" s="19">
+        <v>8.5500000000000007</v>
+      </c>
+      <c r="H233" s="20" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="234" spans="1:8">
+      <c r="A234">
+        <v>233</v>
+      </c>
+      <c r="B234" s="18"/>
+      <c r="C234" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="D234" s="17">
+        <v>46312</v>
+      </c>
+      <c r="E234" s="19">
+        <v>0.73299999999999998</v>
+      </c>
+      <c r="F234" s="19">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G234" s="19">
+        <v>8.49</v>
+      </c>
+      <c r="H234" s="20" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="235" spans="1:8">
+      <c r="A235">
+        <v>234</v>
+      </c>
+      <c r="B235" s="18"/>
+      <c r="C235" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="D235" s="17">
+        <v>46312</v>
+      </c>
+      <c r="E235" s="19">
+        <v>0.72499999999999998</v>
+      </c>
+      <c r="F235" s="19">
+        <v>0.53</v>
+      </c>
+      <c r="G235" s="19">
+        <v>8.14</v>
+      </c>
+      <c r="H235" s="20" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="236" spans="1:8">
+      <c r="A236">
+        <v>235</v>
+      </c>
+      <c r="B236" s="18"/>
+      <c r="C236" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="D236" s="17">
+        <v>46312</v>
+      </c>
+      <c r="E236" s="19">
+        <v>0.73</v>
+      </c>
+      <c r="F236" s="19">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="G236" s="19">
+        <v>8.57</v>
+      </c>
+      <c r="H236" s="20" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="20">
+    <mergeCell ref="B229:B236"/>
+    <mergeCell ref="B209:B228"/>
+    <mergeCell ref="B146:B160"/>
+    <mergeCell ref="B161:B169"/>
+    <mergeCell ref="B170:B178"/>
+    <mergeCell ref="B179:B190"/>
+    <mergeCell ref="B191:B199"/>
+    <mergeCell ref="B200:B208"/>
     <mergeCell ref="B128:B145"/>
     <mergeCell ref="B2:B13"/>
     <mergeCell ref="B14:B22"/>
@@ -10127,13 +10317,6 @@
     <mergeCell ref="B86:B97"/>
     <mergeCell ref="B98:B118"/>
     <mergeCell ref="B119:B127"/>
-    <mergeCell ref="B209:B228"/>
-    <mergeCell ref="B146:B160"/>
-    <mergeCell ref="B161:B169"/>
-    <mergeCell ref="B170:B178"/>
-    <mergeCell ref="B179:B190"/>
-    <mergeCell ref="B191:B199"/>
-    <mergeCell ref="B200:B208"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Upload LF_Ball_Mill_Metallurgical_Report.xlsx via Zeta Client · 263 sel berubah · Data Sampel, Tren Harian
</commit_message>
<xml_diff>
--- a/PRODUKSI/REPORT/LF_Ball_Mill_Metallurgical_Report.xlsx
+++ b/PRODUKSI/REPORT/LF_Ball_Mill_Metallurgical_Report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ramda\Documents\Zeta_Edit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{496E57BD-7A55-4A4F-B224-1C3F11CAC065}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{411F70A5-4552-449A-A4DF-D65884F1C81B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="559" uniqueCount="54">
   <si>
     <t>Periode</t>
   </si>
@@ -226,10 +226,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd\ mmm\ yyyy"/>
+    <numFmt numFmtId="171" formatCode="0.000"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -249,6 +250,26 @@
     <font>
       <b/>
       <sz val="22"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="28"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Carlito"/>
     </font>
   </fonts>
@@ -278,12 +299,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.39997558519241921"/>
+        <fgColor theme="4" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -306,11 +327,48 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -338,24 +396,39 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3453,7 +3526,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
@@ -4489,6 +4562,48 @@
       </c>
       <c r="E40">
         <v>8.41</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
+      <c r="A41" s="2">
+        <v>46313</v>
+      </c>
+      <c r="B41">
+        <f>COUNT('Data Sampel'!D247:D264)</f>
+        <v>18</v>
+      </c>
+      <c r="C41" s="27">
+        <f>AVERAGE('Data Sampel'!E247:E264)</f>
+        <v>0.41022222222222227</v>
+      </c>
+      <c r="D41" s="27">
+        <f>AVERAGE('Data Sampel'!F247:F264)</f>
+        <v>0.34644444444444444</v>
+      </c>
+      <c r="E41" s="27">
+        <f>AVERAGE('Data Sampel'!G247:G264)</f>
+        <v>9.2982222222222219</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8">
+      <c r="A42" s="2">
+        <v>46314</v>
+      </c>
+      <c r="B42">
+        <f>COUNT('Data Sampel'!D265:D269)</f>
+        <v>5</v>
+      </c>
+      <c r="C42" s="27">
+        <f>AVERAGE('Data Sampel'!E265:E269)</f>
+        <v>0.4446</v>
+      </c>
+      <c r="D42" s="27">
+        <f>AVERAGE('Data Sampel'!F265:F269)</f>
+        <v>0.46799999999999997</v>
+      </c>
+      <c r="E42" s="27">
+        <f>AVERAGE('Data Sampel'!G265:G269)</f>
+        <v>11.66</v>
       </c>
     </row>
   </sheetData>
@@ -4652,7 +4767,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:I236"/>
+  <dimension ref="A1:I270"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -4693,7 +4808,7 @@
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="16">
+      <c r="B2" s="15">
         <v>1</v>
       </c>
       <c r="C2" s="5" t="s">
@@ -4719,7 +4834,7 @@
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="16"/>
+      <c r="B3" s="15"/>
       <c r="C3" s="5" t="s">
         <v>37</v>
       </c>
@@ -4743,7 +4858,7 @@
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" s="16"/>
+      <c r="B4" s="15"/>
       <c r="C4" s="5" t="s">
         <v>38</v>
       </c>
@@ -4767,7 +4882,7 @@
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" s="16"/>
+      <c r="B5" s="15"/>
       <c r="C5" s="5" t="s">
         <v>39</v>
       </c>
@@ -4791,7 +4906,7 @@
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" s="16"/>
+      <c r="B6" s="15"/>
       <c r="C6" s="5" t="s">
         <v>40</v>
       </c>
@@ -4815,7 +4930,7 @@
       <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7" s="16"/>
+      <c r="B7" s="15"/>
       <c r="C7" s="5" t="s">
         <v>41</v>
       </c>
@@ -4839,7 +4954,7 @@
       <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8" s="16"/>
+      <c r="B8" s="15"/>
       <c r="C8" s="5" t="s">
         <v>36</v>
       </c>
@@ -4863,7 +4978,7 @@
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" s="16"/>
+      <c r="B9" s="15"/>
       <c r="C9" s="5" t="s">
         <v>37</v>
       </c>
@@ -4887,7 +5002,7 @@
       <c r="A10">
         <v>9</v>
       </c>
-      <c r="B10" s="16"/>
+      <c r="B10" s="15"/>
       <c r="C10" s="5" t="s">
         <v>38</v>
       </c>
@@ -4911,7 +5026,7 @@
       <c r="A11">
         <v>10</v>
       </c>
-      <c r="B11" s="16"/>
+      <c r="B11" s="15"/>
       <c r="C11" s="5" t="s">
         <v>39</v>
       </c>
@@ -4935,7 +5050,7 @@
       <c r="A12">
         <v>11</v>
       </c>
-      <c r="B12" s="16"/>
+      <c r="B12" s="15"/>
       <c r="C12" s="5" t="s">
         <v>40</v>
       </c>
@@ -4959,7 +5074,7 @@
       <c r="A13">
         <v>12</v>
       </c>
-      <c r="B13" s="16"/>
+      <c r="B13" s="15"/>
       <c r="C13" s="5" t="s">
         <v>41</v>
       </c>
@@ -4983,7 +5098,7 @@
       <c r="A14">
         <v>13</v>
       </c>
-      <c r="B14" s="15">
+      <c r="B14" s="16">
         <v>2</v>
       </c>
       <c r="C14" s="7" t="s">
@@ -5009,7 +5124,7 @@
       <c r="A15">
         <v>14</v>
       </c>
-      <c r="B15" s="15"/>
+      <c r="B15" s="16"/>
       <c r="C15" s="7" t="s">
         <v>37</v>
       </c>
@@ -5033,7 +5148,7 @@
       <c r="A16">
         <v>15</v>
       </c>
-      <c r="B16" s="15"/>
+      <c r="B16" s="16"/>
       <c r="C16" s="7" t="s">
         <v>38</v>
       </c>
@@ -5057,7 +5172,7 @@
       <c r="A17">
         <v>16</v>
       </c>
-      <c r="B17" s="15"/>
+      <c r="B17" s="16"/>
       <c r="C17" s="7" t="s">
         <v>39</v>
       </c>
@@ -5081,7 +5196,7 @@
       <c r="A18">
         <v>17</v>
       </c>
-      <c r="B18" s="15"/>
+      <c r="B18" s="16"/>
       <c r="C18" s="7" t="s">
         <v>40</v>
       </c>
@@ -5105,7 +5220,7 @@
       <c r="A19">
         <v>18</v>
       </c>
-      <c r="B19" s="15"/>
+      <c r="B19" s="16"/>
       <c r="C19" s="7" t="s">
         <v>41</v>
       </c>
@@ -5129,7 +5244,7 @@
       <c r="A20">
         <v>19</v>
       </c>
-      <c r="B20" s="15"/>
+      <c r="B20" s="16"/>
       <c r="C20" s="7" t="s">
         <v>36</v>
       </c>
@@ -5153,7 +5268,7 @@
       <c r="A21">
         <v>20</v>
       </c>
-      <c r="B21" s="15"/>
+      <c r="B21" s="16"/>
       <c r="C21" s="7" t="s">
         <v>37</v>
       </c>
@@ -5177,7 +5292,7 @@
       <c r="A22">
         <v>21</v>
       </c>
-      <c r="B22" s="15"/>
+      <c r="B22" s="16"/>
       <c r="C22" s="7" t="s">
         <v>38</v>
       </c>
@@ -5201,7 +5316,7 @@
       <c r="A23">
         <v>22</v>
       </c>
-      <c r="B23" s="16">
+      <c r="B23" s="15">
         <v>3</v>
       </c>
       <c r="C23" s="5" t="s">
@@ -5227,7 +5342,7 @@
       <c r="A24">
         <v>23</v>
       </c>
-      <c r="B24" s="16"/>
+      <c r="B24" s="15"/>
       <c r="C24" s="5" t="s">
         <v>40</v>
       </c>
@@ -5251,7 +5366,7 @@
       <c r="A25">
         <v>24</v>
       </c>
-      <c r="B25" s="16"/>
+      <c r="B25" s="15"/>
       <c r="C25" s="5" t="s">
         <v>41</v>
       </c>
@@ -5275,7 +5390,7 @@
       <c r="A26">
         <v>25</v>
       </c>
-      <c r="B26" s="16"/>
+      <c r="B26" s="15"/>
       <c r="C26" s="5" t="s">
         <v>36</v>
       </c>
@@ -5299,7 +5414,7 @@
       <c r="A27">
         <v>26</v>
       </c>
-      <c r="B27" s="16"/>
+      <c r="B27" s="15"/>
       <c r="C27" s="5" t="s">
         <v>37</v>
       </c>
@@ -5323,7 +5438,7 @@
       <c r="A28">
         <v>27</v>
       </c>
-      <c r="B28" s="16"/>
+      <c r="B28" s="15"/>
       <c r="C28" s="5" t="s">
         <v>38</v>
       </c>
@@ -5347,7 +5462,7 @@
       <c r="A29">
         <v>28</v>
       </c>
-      <c r="B29" s="16"/>
+      <c r="B29" s="15"/>
       <c r="C29" s="5" t="s">
         <v>39</v>
       </c>
@@ -5371,7 +5486,7 @@
       <c r="A30">
         <v>29</v>
       </c>
-      <c r="B30" s="16"/>
+      <c r="B30" s="15"/>
       <c r="C30" s="5" t="s">
         <v>40</v>
       </c>
@@ -5395,7 +5510,7 @@
       <c r="A31">
         <v>30</v>
       </c>
-      <c r="B31" s="16"/>
+      <c r="B31" s="15"/>
       <c r="C31" s="5" t="s">
         <v>41</v>
       </c>
@@ -5419,7 +5534,7 @@
       <c r="A32">
         <v>31</v>
       </c>
-      <c r="B32" s="16"/>
+      <c r="B32" s="15"/>
       <c r="C32" s="5" t="s">
         <v>36</v>
       </c>
@@ -5443,7 +5558,7 @@
       <c r="A33">
         <v>32</v>
       </c>
-      <c r="B33" s="16"/>
+      <c r="B33" s="15"/>
       <c r="C33" s="5" t="s">
         <v>37</v>
       </c>
@@ -5467,7 +5582,7 @@
       <c r="A34">
         <v>33</v>
       </c>
-      <c r="B34" s="16"/>
+      <c r="B34" s="15"/>
       <c r="C34" s="5" t="s">
         <v>38</v>
       </c>
@@ -5491,7 +5606,7 @@
       <c r="A35">
         <v>34</v>
       </c>
-      <c r="B35" s="15">
+      <c r="B35" s="16">
         <v>4</v>
       </c>
       <c r="C35" s="7" t="s">
@@ -5517,7 +5632,7 @@
       <c r="A36">
         <v>35</v>
       </c>
-      <c r="B36" s="15"/>
+      <c r="B36" s="16"/>
       <c r="C36" s="7" t="s">
         <v>40</v>
       </c>
@@ -5541,7 +5656,7 @@
       <c r="A37">
         <v>36</v>
       </c>
-      <c r="B37" s="15"/>
+      <c r="B37" s="16"/>
       <c r="C37" s="7" t="s">
         <v>41</v>
       </c>
@@ -5565,7 +5680,7 @@
       <c r="A38">
         <v>37</v>
       </c>
-      <c r="B38" s="15"/>
+      <c r="B38" s="16"/>
       <c r="C38" s="7" t="s">
         <v>36</v>
       </c>
@@ -5589,7 +5704,7 @@
       <c r="A39">
         <v>38</v>
       </c>
-      <c r="B39" s="15"/>
+      <c r="B39" s="16"/>
       <c r="C39" s="7" t="s">
         <v>37</v>
       </c>
@@ -5613,7 +5728,7 @@
       <c r="A40">
         <v>39</v>
       </c>
-      <c r="B40" s="15"/>
+      <c r="B40" s="16"/>
       <c r="C40" s="7" t="s">
         <v>38</v>
       </c>
@@ -5637,7 +5752,7 @@
       <c r="A41">
         <v>40</v>
       </c>
-      <c r="B41" s="15"/>
+      <c r="B41" s="16"/>
       <c r="C41" s="7" t="s">
         <v>39</v>
       </c>
@@ -5661,7 +5776,7 @@
       <c r="A42">
         <v>41</v>
       </c>
-      <c r="B42" s="15"/>
+      <c r="B42" s="16"/>
       <c r="C42" s="7" t="s">
         <v>40</v>
       </c>
@@ -5685,7 +5800,7 @@
       <c r="A43">
         <v>42</v>
       </c>
-      <c r="B43" s="15"/>
+      <c r="B43" s="16"/>
       <c r="C43" s="7" t="s">
         <v>41</v>
       </c>
@@ -5709,7 +5824,7 @@
       <c r="A44">
         <v>43</v>
       </c>
-      <c r="B44" s="15"/>
+      <c r="B44" s="16"/>
       <c r="C44" s="7" t="s">
         <v>36</v>
       </c>
@@ -5733,7 +5848,7 @@
       <c r="A45">
         <v>44</v>
       </c>
-      <c r="B45" s="15"/>
+      <c r="B45" s="16"/>
       <c r="C45" s="7" t="s">
         <v>37</v>
       </c>
@@ -5757,7 +5872,7 @@
       <c r="A46">
         <v>45</v>
       </c>
-      <c r="B46" s="15"/>
+      <c r="B46" s="16"/>
       <c r="C46" s="7" t="s">
         <v>38</v>
       </c>
@@ -5781,7 +5896,7 @@
       <c r="A47">
         <v>46</v>
       </c>
-      <c r="B47" s="15"/>
+      <c r="B47" s="16"/>
       <c r="C47" s="7" t="s">
         <v>39</v>
       </c>
@@ -5799,7 +5914,7 @@
       <c r="A48">
         <v>47</v>
       </c>
-      <c r="B48" s="15"/>
+      <c r="B48" s="16"/>
       <c r="C48" s="7" t="s">
         <v>40</v>
       </c>
@@ -5817,7 +5932,7 @@
       <c r="A49">
         <v>48</v>
       </c>
-      <c r="B49" s="15"/>
+      <c r="B49" s="16"/>
       <c r="C49" s="7" t="s">
         <v>41</v>
       </c>
@@ -5835,7 +5950,7 @@
       <c r="A50">
         <v>49</v>
       </c>
-      <c r="B50" s="16">
+      <c r="B50" s="15">
         <v>5</v>
       </c>
       <c r="C50" s="5" t="s">
@@ -5861,7 +5976,7 @@
       <c r="A51">
         <v>50</v>
       </c>
-      <c r="B51" s="16"/>
+      <c r="B51" s="15"/>
       <c r="C51" s="5" t="s">
         <v>37</v>
       </c>
@@ -5885,7 +6000,7 @@
       <c r="A52">
         <v>51</v>
       </c>
-      <c r="B52" s="16"/>
+      <c r="B52" s="15"/>
       <c r="C52" s="5" t="s">
         <v>38</v>
       </c>
@@ -5909,7 +6024,7 @@
       <c r="A53">
         <v>52</v>
       </c>
-      <c r="B53" s="16"/>
+      <c r="B53" s="15"/>
       <c r="C53" s="5" t="s">
         <v>39</v>
       </c>
@@ -5933,7 +6048,7 @@
       <c r="A54">
         <v>53</v>
       </c>
-      <c r="B54" s="16"/>
+      <c r="B54" s="15"/>
       <c r="C54" s="5" t="s">
         <v>40</v>
       </c>
@@ -5957,7 +6072,7 @@
       <c r="A55">
         <v>54</v>
       </c>
-      <c r="B55" s="16"/>
+      <c r="B55" s="15"/>
       <c r="C55" s="5" t="s">
         <v>41</v>
       </c>
@@ -5981,7 +6096,7 @@
       <c r="A56">
         <v>55</v>
       </c>
-      <c r="B56" s="16"/>
+      <c r="B56" s="15"/>
       <c r="C56" s="5" t="s">
         <v>36</v>
       </c>
@@ -6005,7 +6120,7 @@
       <c r="A57">
         <v>56</v>
       </c>
-      <c r="B57" s="16"/>
+      <c r="B57" s="15"/>
       <c r="C57" s="5" t="s">
         <v>37</v>
       </c>
@@ -6029,7 +6144,7 @@
       <c r="A58">
         <v>57</v>
       </c>
-      <c r="B58" s="16"/>
+      <c r="B58" s="15"/>
       <c r="C58" s="5" t="s">
         <v>38</v>
       </c>
@@ -6053,7 +6168,7 @@
       <c r="A59">
         <v>58</v>
       </c>
-      <c r="B59" s="15">
+      <c r="B59" s="16">
         <v>6</v>
       </c>
       <c r="C59" s="7" t="s">
@@ -6079,7 +6194,7 @@
       <c r="A60">
         <v>59</v>
       </c>
-      <c r="B60" s="15"/>
+      <c r="B60" s="16"/>
       <c r="C60" s="7" t="s">
         <v>40</v>
       </c>
@@ -6103,7 +6218,7 @@
       <c r="A61">
         <v>60</v>
       </c>
-      <c r="B61" s="15"/>
+      <c r="B61" s="16"/>
       <c r="C61" s="7" t="s">
         <v>41</v>
       </c>
@@ -6127,7 +6242,7 @@
       <c r="A62">
         <v>61</v>
       </c>
-      <c r="B62" s="15"/>
+      <c r="B62" s="16"/>
       <c r="C62" s="7" t="s">
         <v>36</v>
       </c>
@@ -6151,7 +6266,7 @@
       <c r="A63">
         <v>62</v>
       </c>
-      <c r="B63" s="15"/>
+      <c r="B63" s="16"/>
       <c r="C63" s="7" t="s">
         <v>37</v>
       </c>
@@ -6175,7 +6290,7 @@
       <c r="A64">
         <v>63</v>
       </c>
-      <c r="B64" s="15"/>
+      <c r="B64" s="16"/>
       <c r="C64" s="7" t="s">
         <v>38</v>
       </c>
@@ -6199,7 +6314,7 @@
       <c r="A65">
         <v>64</v>
       </c>
-      <c r="B65" s="16">
+      <c r="B65" s="15">
         <v>7</v>
       </c>
       <c r="C65" s="5" t="s">
@@ -6225,7 +6340,7 @@
       <c r="A66">
         <v>65</v>
       </c>
-      <c r="B66" s="16"/>
+      <c r="B66" s="15"/>
       <c r="C66" s="5" t="s">
         <v>40</v>
       </c>
@@ -6249,7 +6364,7 @@
       <c r="A67">
         <v>66</v>
       </c>
-      <c r="B67" s="16"/>
+      <c r="B67" s="15"/>
       <c r="C67" s="5" t="s">
         <v>41</v>
       </c>
@@ -6273,7 +6388,7 @@
       <c r="A68">
         <v>67</v>
       </c>
-      <c r="B68" s="16"/>
+      <c r="B68" s="15"/>
       <c r="C68" s="5" t="s">
         <v>36</v>
       </c>
@@ -6297,7 +6412,7 @@
       <c r="A69">
         <v>68</v>
       </c>
-      <c r="B69" s="16"/>
+      <c r="B69" s="15"/>
       <c r="C69" s="5" t="s">
         <v>37</v>
       </c>
@@ -6321,7 +6436,7 @@
       <c r="A70">
         <v>69</v>
       </c>
-      <c r="B70" s="16"/>
+      <c r="B70" s="15"/>
       <c r="C70" s="5" t="s">
         <v>38</v>
       </c>
@@ -6345,7 +6460,7 @@
       <c r="A71">
         <v>70</v>
       </c>
-      <c r="B71" s="16"/>
+      <c r="B71" s="15"/>
       <c r="C71" s="5" t="s">
         <v>39</v>
       </c>
@@ -6369,7 +6484,7 @@
       <c r="A72">
         <v>71</v>
       </c>
-      <c r="B72" s="16"/>
+      <c r="B72" s="15"/>
       <c r="C72" s="5" t="s">
         <v>40</v>
       </c>
@@ -6393,7 +6508,7 @@
       <c r="A73">
         <v>72</v>
       </c>
-      <c r="B73" s="16"/>
+      <c r="B73" s="15"/>
       <c r="C73" s="5" t="s">
         <v>41</v>
       </c>
@@ -6417,7 +6532,7 @@
       <c r="A74">
         <v>73</v>
       </c>
-      <c r="B74" s="15">
+      <c r="B74" s="16">
         <v>8</v>
       </c>
       <c r="C74" s="7" t="s">
@@ -6443,7 +6558,7 @@
       <c r="A75">
         <v>74</v>
       </c>
-      <c r="B75" s="15"/>
+      <c r="B75" s="16"/>
       <c r="C75" s="7" t="s">
         <v>37</v>
       </c>
@@ -6467,7 +6582,7 @@
       <c r="A76">
         <v>75</v>
       </c>
-      <c r="B76" s="15"/>
+      <c r="B76" s="16"/>
       <c r="C76" s="7" t="s">
         <v>38</v>
       </c>
@@ -6491,7 +6606,7 @@
       <c r="A77">
         <v>76</v>
       </c>
-      <c r="B77" s="15"/>
+      <c r="B77" s="16"/>
       <c r="C77" s="7" t="s">
         <v>39</v>
       </c>
@@ -6515,7 +6630,7 @@
       <c r="A78">
         <v>77</v>
       </c>
-      <c r="B78" s="15"/>
+      <c r="B78" s="16"/>
       <c r="C78" s="7" t="s">
         <v>40</v>
       </c>
@@ -6539,7 +6654,7 @@
       <c r="A79">
         <v>78</v>
       </c>
-      <c r="B79" s="15"/>
+      <c r="B79" s="16"/>
       <c r="C79" s="7" t="s">
         <v>41</v>
       </c>
@@ -6563,7 +6678,7 @@
       <c r="A80">
         <v>79</v>
       </c>
-      <c r="B80" s="15"/>
+      <c r="B80" s="16"/>
       <c r="C80" s="7" t="s">
         <v>36</v>
       </c>
@@ -6587,7 +6702,7 @@
       <c r="A81">
         <v>80</v>
       </c>
-      <c r="B81" s="15"/>
+      <c r="B81" s="16"/>
       <c r="C81" s="7" t="s">
         <v>37</v>
       </c>
@@ -6611,7 +6726,7 @@
       <c r="A82">
         <v>81</v>
       </c>
-      <c r="B82" s="15"/>
+      <c r="B82" s="16"/>
       <c r="C82" s="7" t="s">
         <v>38</v>
       </c>
@@ -6635,7 +6750,7 @@
       <c r="A83">
         <v>82</v>
       </c>
-      <c r="B83" s="15"/>
+      <c r="B83" s="16"/>
       <c r="C83" s="7" t="s">
         <v>39</v>
       </c>
@@ -6659,7 +6774,7 @@
       <c r="A84">
         <v>83</v>
       </c>
-      <c r="B84" s="15"/>
+      <c r="B84" s="16"/>
       <c r="C84" s="7" t="s">
         <v>40</v>
       </c>
@@ -6683,7 +6798,7 @@
       <c r="A85">
         <v>84</v>
       </c>
-      <c r="B85" s="15"/>
+      <c r="B85" s="16"/>
       <c r="C85" s="7" t="s">
         <v>41</v>
       </c>
@@ -6707,7 +6822,7 @@
       <c r="A86">
         <v>85</v>
       </c>
-      <c r="B86" s="16">
+      <c r="B86" s="15">
         <v>9</v>
       </c>
       <c r="C86" s="5" t="s">
@@ -6733,7 +6848,7 @@
       <c r="A87">
         <v>86</v>
       </c>
-      <c r="B87" s="16"/>
+      <c r="B87" s="15"/>
       <c r="C87" s="5" t="s">
         <v>37</v>
       </c>
@@ -6757,7 +6872,7 @@
       <c r="A88">
         <v>87</v>
       </c>
-      <c r="B88" s="16"/>
+      <c r="B88" s="15"/>
       <c r="C88" s="5" t="s">
         <v>38</v>
       </c>
@@ -6781,7 +6896,7 @@
       <c r="A89">
         <v>88</v>
       </c>
-      <c r="B89" s="16"/>
+      <c r="B89" s="15"/>
       <c r="C89" s="5" t="s">
         <v>39</v>
       </c>
@@ -6805,7 +6920,7 @@
       <c r="A90">
         <v>89</v>
       </c>
-      <c r="B90" s="16"/>
+      <c r="B90" s="15"/>
       <c r="C90" s="5" t="s">
         <v>40</v>
       </c>
@@ -6829,7 +6944,7 @@
       <c r="A91">
         <v>90</v>
       </c>
-      <c r="B91" s="16"/>
+      <c r="B91" s="15"/>
       <c r="C91" s="5" t="s">
         <v>41</v>
       </c>
@@ -6853,7 +6968,7 @@
       <c r="A92">
         <v>91</v>
       </c>
-      <c r="B92" s="16"/>
+      <c r="B92" s="15"/>
       <c r="C92" s="5" t="s">
         <v>36</v>
       </c>
@@ -6877,7 +6992,7 @@
       <c r="A93">
         <v>92</v>
       </c>
-      <c r="B93" s="16"/>
+      <c r="B93" s="15"/>
       <c r="C93" s="5" t="s">
         <v>37</v>
       </c>
@@ -6901,7 +7016,7 @@
       <c r="A94">
         <v>93</v>
       </c>
-      <c r="B94" s="16"/>
+      <c r="B94" s="15"/>
       <c r="C94" s="5" t="s">
         <v>38</v>
       </c>
@@ -6925,7 +7040,7 @@
       <c r="A95">
         <v>94</v>
       </c>
-      <c r="B95" s="16"/>
+      <c r="B95" s="15"/>
       <c r="C95" s="5" t="s">
         <v>39</v>
       </c>
@@ -6949,7 +7064,7 @@
       <c r="A96">
         <v>95</v>
       </c>
-      <c r="B96" s="16"/>
+      <c r="B96" s="15"/>
       <c r="C96" s="5" t="s">
         <v>40</v>
       </c>
@@ -6973,7 +7088,7 @@
       <c r="A97">
         <v>96</v>
       </c>
-      <c r="B97" s="16"/>
+      <c r="B97" s="15"/>
       <c r="C97" s="5" t="s">
         <v>41</v>
       </c>
@@ -6997,7 +7112,7 @@
       <c r="A98">
         <v>97</v>
       </c>
-      <c r="B98" s="15">
+      <c r="B98" s="16">
         <v>10</v>
       </c>
       <c r="C98" s="7" t="s">
@@ -7023,7 +7138,7 @@
       <c r="A99">
         <v>98</v>
       </c>
-      <c r="B99" s="15"/>
+      <c r="B99" s="16"/>
       <c r="C99" s="7" t="s">
         <v>37</v>
       </c>
@@ -7047,7 +7162,7 @@
       <c r="A100">
         <v>99</v>
       </c>
-      <c r="B100" s="15"/>
+      <c r="B100" s="16"/>
       <c r="C100" s="7" t="s">
         <v>38</v>
       </c>
@@ -7071,7 +7186,7 @@
       <c r="A101">
         <v>100</v>
       </c>
-      <c r="B101" s="15"/>
+      <c r="B101" s="16"/>
       <c r="C101" s="7" t="s">
         <v>39</v>
       </c>
@@ -7095,7 +7210,7 @@
       <c r="A102">
         <v>101</v>
       </c>
-      <c r="B102" s="15"/>
+      <c r="B102" s="16"/>
       <c r="C102" s="7" t="s">
         <v>40</v>
       </c>
@@ -7119,7 +7234,7 @@
       <c r="A103">
         <v>102</v>
       </c>
-      <c r="B103" s="15"/>
+      <c r="B103" s="16"/>
       <c r="C103" s="7" t="s">
         <v>41</v>
       </c>
@@ -7143,7 +7258,7 @@
       <c r="A104">
         <v>103</v>
       </c>
-      <c r="B104" s="15"/>
+      <c r="B104" s="16"/>
       <c r="C104" s="7" t="s">
         <v>36</v>
       </c>
@@ -7167,7 +7282,7 @@
       <c r="A105">
         <v>104</v>
       </c>
-      <c r="B105" s="15"/>
+      <c r="B105" s="16"/>
       <c r="C105" s="7" t="s">
         <v>37</v>
       </c>
@@ -7191,7 +7306,7 @@
       <c r="A106">
         <v>105</v>
       </c>
-      <c r="B106" s="15"/>
+      <c r="B106" s="16"/>
       <c r="C106" s="7" t="s">
         <v>38</v>
       </c>
@@ -7215,7 +7330,7 @@
       <c r="A107">
         <v>106</v>
       </c>
-      <c r="B107" s="15"/>
+      <c r="B107" s="16"/>
       <c r="C107" s="7" t="s">
         <v>39</v>
       </c>
@@ -7239,7 +7354,7 @@
       <c r="A108">
         <v>107</v>
       </c>
-      <c r="B108" s="15"/>
+      <c r="B108" s="16"/>
       <c r="C108" s="7" t="s">
         <v>40</v>
       </c>
@@ -7263,7 +7378,7 @@
       <c r="A109">
         <v>108</v>
       </c>
-      <c r="B109" s="15"/>
+      <c r="B109" s="16"/>
       <c r="C109" s="7" t="s">
         <v>41</v>
       </c>
@@ -7287,7 +7402,7 @@
       <c r="A110">
         <v>109</v>
       </c>
-      <c r="B110" s="15"/>
+      <c r="B110" s="16"/>
       <c r="C110" s="7" t="s">
         <v>36</v>
       </c>
@@ -7311,7 +7426,7 @@
       <c r="A111">
         <v>110</v>
       </c>
-      <c r="B111" s="15"/>
+      <c r="B111" s="16"/>
       <c r="C111" s="7" t="s">
         <v>37</v>
       </c>
@@ -7335,7 +7450,7 @@
       <c r="A112">
         <v>111</v>
       </c>
-      <c r="B112" s="15"/>
+      <c r="B112" s="16"/>
       <c r="C112" s="7" t="s">
         <v>38</v>
       </c>
@@ -7359,7 +7474,7 @@
       <c r="A113">
         <v>112</v>
       </c>
-      <c r="B113" s="15"/>
+      <c r="B113" s="16"/>
       <c r="C113" s="7" t="s">
         <v>39</v>
       </c>
@@ -7383,7 +7498,7 @@
       <c r="A114">
         <v>113</v>
       </c>
-      <c r="B114" s="15"/>
+      <c r="B114" s="16"/>
       <c r="C114" s="7" t="s">
         <v>40</v>
       </c>
@@ -7407,7 +7522,7 @@
       <c r="A115">
         <v>114</v>
       </c>
-      <c r="B115" s="15"/>
+      <c r="B115" s="16"/>
       <c r="C115" s="7" t="s">
         <v>41</v>
       </c>
@@ -7431,7 +7546,7 @@
       <c r="A116">
         <v>115</v>
       </c>
-      <c r="B116" s="15"/>
+      <c r="B116" s="16"/>
       <c r="C116" s="7" t="s">
         <v>36</v>
       </c>
@@ -7455,7 +7570,7 @@
       <c r="A117">
         <v>116</v>
       </c>
-      <c r="B117" s="15"/>
+      <c r="B117" s="16"/>
       <c r="C117" s="7" t="s">
         <v>37</v>
       </c>
@@ -7479,7 +7594,7 @@
       <c r="A118">
         <v>117</v>
       </c>
-      <c r="B118" s="15"/>
+      <c r="B118" s="16"/>
       <c r="C118" s="7" t="s">
         <v>38</v>
       </c>
@@ -7503,7 +7618,7 @@
       <c r="A119">
         <v>118</v>
       </c>
-      <c r="B119" s="16">
+      <c r="B119" s="15">
         <v>11</v>
       </c>
       <c r="C119" s="5" t="s">
@@ -7529,7 +7644,7 @@
       <c r="A120">
         <v>119</v>
       </c>
-      <c r="B120" s="16"/>
+      <c r="B120" s="15"/>
       <c r="C120" s="5" t="s">
         <v>40</v>
       </c>
@@ -7553,7 +7668,7 @@
       <c r="A121">
         <v>120</v>
       </c>
-      <c r="B121" s="16"/>
+      <c r="B121" s="15"/>
       <c r="C121" s="5" t="s">
         <v>41</v>
       </c>
@@ -7577,7 +7692,7 @@
       <c r="A122">
         <v>121</v>
       </c>
-      <c r="B122" s="16"/>
+      <c r="B122" s="15"/>
       <c r="C122" s="5" t="s">
         <v>36</v>
       </c>
@@ -7601,7 +7716,7 @@
       <c r="A123">
         <v>122</v>
       </c>
-      <c r="B123" s="16"/>
+      <c r="B123" s="15"/>
       <c r="C123" s="5" t="s">
         <v>37</v>
       </c>
@@ -7625,7 +7740,7 @@
       <c r="A124">
         <v>123</v>
       </c>
-      <c r="B124" s="16"/>
+      <c r="B124" s="15"/>
       <c r="C124" s="5" t="s">
         <v>38</v>
       </c>
@@ -7649,7 +7764,7 @@
       <c r="A125">
         <v>124</v>
       </c>
-      <c r="B125" s="16"/>
+      <c r="B125" s="15"/>
       <c r="C125" s="5" t="s">
         <v>39</v>
       </c>
@@ -7667,7 +7782,7 @@
       <c r="A126">
         <v>125</v>
       </c>
-      <c r="B126" s="16"/>
+      <c r="B126" s="15"/>
       <c r="C126" s="5" t="s">
         <v>40</v>
       </c>
@@ -7685,7 +7800,7 @@
       <c r="A127">
         <v>126</v>
       </c>
-      <c r="B127" s="16"/>
+      <c r="B127" s="15"/>
       <c r="C127" s="5" t="s">
         <v>41</v>
       </c>
@@ -7703,7 +7818,7 @@
       <c r="A128">
         <v>127</v>
       </c>
-      <c r="B128" s="15">
+      <c r="B128" s="16">
         <v>12</v>
       </c>
       <c r="C128" s="7" t="s">
@@ -7729,7 +7844,7 @@
       <c r="A129">
         <v>128</v>
       </c>
-      <c r="B129" s="15"/>
+      <c r="B129" s="16"/>
       <c r="C129" s="7" t="s">
         <v>37</v>
       </c>
@@ -7753,7 +7868,7 @@
       <c r="A130">
         <v>129</v>
       </c>
-      <c r="B130" s="15"/>
+      <c r="B130" s="16"/>
       <c r="C130" s="7" t="s">
         <v>38</v>
       </c>
@@ -7777,7 +7892,7 @@
       <c r="A131">
         <v>130</v>
       </c>
-      <c r="B131" s="15"/>
+      <c r="B131" s="16"/>
       <c r="C131" s="7" t="s">
         <v>39</v>
       </c>
@@ -7801,7 +7916,7 @@
       <c r="A132">
         <v>131</v>
       </c>
-      <c r="B132" s="15"/>
+      <c r="B132" s="16"/>
       <c r="C132" s="7" t="s">
         <v>40</v>
       </c>
@@ -7825,7 +7940,7 @@
       <c r="A133">
         <v>132</v>
       </c>
-      <c r="B133" s="15"/>
+      <c r="B133" s="16"/>
       <c r="C133" s="7" t="s">
         <v>41</v>
       </c>
@@ -7849,7 +7964,7 @@
       <c r="A134">
         <v>133</v>
       </c>
-      <c r="B134" s="15"/>
+      <c r="B134" s="16"/>
       <c r="C134" s="7" t="s">
         <v>36</v>
       </c>
@@ -7873,7 +7988,7 @@
       <c r="A135">
         <v>134</v>
       </c>
-      <c r="B135" s="15"/>
+      <c r="B135" s="16"/>
       <c r="C135" s="7" t="s">
         <v>37</v>
       </c>
@@ -7897,7 +8012,7 @@
       <c r="A136">
         <v>135</v>
       </c>
-      <c r="B136" s="15"/>
+      <c r="B136" s="16"/>
       <c r="C136" s="7" t="s">
         <v>38</v>
       </c>
@@ -7921,7 +8036,7 @@
       <c r="A137">
         <v>136</v>
       </c>
-      <c r="B137" s="15"/>
+      <c r="B137" s="16"/>
       <c r="C137" s="7" t="s">
         <v>39</v>
       </c>
@@ -7945,7 +8060,7 @@
       <c r="A138">
         <v>137</v>
       </c>
-      <c r="B138" s="15"/>
+      <c r="B138" s="16"/>
       <c r="C138" s="7" t="s">
         <v>40</v>
       </c>
@@ -7969,7 +8084,7 @@
       <c r="A139">
         <v>138</v>
       </c>
-      <c r="B139" s="15"/>
+      <c r="B139" s="16"/>
       <c r="C139" s="7" t="s">
         <v>41</v>
       </c>
@@ -7993,7 +8108,7 @@
       <c r="A140">
         <v>139</v>
       </c>
-      <c r="B140" s="15"/>
+      <c r="B140" s="16"/>
       <c r="C140" s="7" t="s">
         <v>36</v>
       </c>
@@ -8017,7 +8132,7 @@
       <c r="A141">
         <v>140</v>
       </c>
-      <c r="B141" s="15"/>
+      <c r="B141" s="16"/>
       <c r="C141" s="7" t="s">
         <v>37</v>
       </c>
@@ -8041,7 +8156,7 @@
       <c r="A142">
         <v>141</v>
       </c>
-      <c r="B142" s="15"/>
+      <c r="B142" s="16"/>
       <c r="C142" s="7" t="s">
         <v>38</v>
       </c>
@@ -8065,7 +8180,7 @@
       <c r="A143">
         <v>142</v>
       </c>
-      <c r="B143" s="15"/>
+      <c r="B143" s="16"/>
       <c r="C143" s="7" t="s">
         <v>39</v>
       </c>
@@ -8089,7 +8204,7 @@
       <c r="A144">
         <v>143</v>
       </c>
-      <c r="B144" s="15"/>
+      <c r="B144" s="16"/>
       <c r="C144" s="7" t="s">
         <v>40</v>
       </c>
@@ -8113,7 +8228,7 @@
       <c r="A145">
         <v>144</v>
       </c>
-      <c r="B145" s="15"/>
+      <c r="B145" s="16"/>
       <c r="C145" s="7" t="s">
         <v>41</v>
       </c>
@@ -8137,7 +8252,7 @@
       <c r="A146">
         <v>145</v>
       </c>
-      <c r="B146" s="16">
+      <c r="B146" s="15">
         <v>13</v>
       </c>
       <c r="C146" s="5" t="s">
@@ -8163,7 +8278,7 @@
       <c r="A147">
         <v>146</v>
       </c>
-      <c r="B147" s="16"/>
+      <c r="B147" s="15"/>
       <c r="C147" s="5" t="s">
         <v>40</v>
       </c>
@@ -8187,7 +8302,7 @@
       <c r="A148">
         <v>147</v>
       </c>
-      <c r="B148" s="16"/>
+      <c r="B148" s="15"/>
       <c r="C148" s="5" t="s">
         <v>41</v>
       </c>
@@ -8211,7 +8326,7 @@
       <c r="A149">
         <v>148</v>
       </c>
-      <c r="B149" s="16"/>
+      <c r="B149" s="15"/>
       <c r="C149" s="5" t="s">
         <v>36</v>
       </c>
@@ -8235,7 +8350,7 @@
       <c r="A150">
         <v>149</v>
       </c>
-      <c r="B150" s="16"/>
+      <c r="B150" s="15"/>
       <c r="C150" s="5" t="s">
         <v>37</v>
       </c>
@@ -8259,7 +8374,7 @@
       <c r="A151">
         <v>150</v>
       </c>
-      <c r="B151" s="16"/>
+      <c r="B151" s="15"/>
       <c r="C151" s="5" t="s">
         <v>38</v>
       </c>
@@ -8283,7 +8398,7 @@
       <c r="A152">
         <v>151</v>
       </c>
-      <c r="B152" s="16"/>
+      <c r="B152" s="15"/>
       <c r="C152" s="5" t="s">
         <v>39</v>
       </c>
@@ -8307,7 +8422,7 @@
       <c r="A153">
         <v>152</v>
       </c>
-      <c r="B153" s="16"/>
+      <c r="B153" s="15"/>
       <c r="C153" s="5" t="s">
         <v>40</v>
       </c>
@@ -8331,7 +8446,7 @@
       <c r="A154">
         <v>153</v>
       </c>
-      <c r="B154" s="16"/>
+      <c r="B154" s="15"/>
       <c r="C154" s="5" t="s">
         <v>41</v>
       </c>
@@ -8355,7 +8470,7 @@
       <c r="A155">
         <v>154</v>
       </c>
-      <c r="B155" s="16"/>
+      <c r="B155" s="15"/>
       <c r="C155" s="5" t="s">
         <v>36</v>
       </c>
@@ -8383,7 +8498,7 @@
       <c r="A156">
         <v>155</v>
       </c>
-      <c r="B156" s="16"/>
+      <c r="B156" s="15"/>
       <c r="C156" s="5" t="s">
         <v>37</v>
       </c>
@@ -8407,7 +8522,7 @@
       <c r="A157">
         <v>156</v>
       </c>
-      <c r="B157" s="16"/>
+      <c r="B157" s="15"/>
       <c r="C157" s="5" t="s">
         <v>38</v>
       </c>
@@ -8431,7 +8546,7 @@
       <c r="A158">
         <v>157</v>
       </c>
-      <c r="B158" s="16"/>
+      <c r="B158" s="15"/>
       <c r="C158" s="5" t="s">
         <v>39</v>
       </c>
@@ -8455,7 +8570,7 @@
       <c r="A159">
         <v>158</v>
       </c>
-      <c r="B159" s="16"/>
+      <c r="B159" s="15"/>
       <c r="C159" s="5" t="s">
         <v>40</v>
       </c>
@@ -8479,7 +8594,7 @@
       <c r="A160">
         <v>159</v>
       </c>
-      <c r="B160" s="16"/>
+      <c r="B160" s="15"/>
       <c r="C160" s="5" t="s">
         <v>41</v>
       </c>
@@ -8503,7 +8618,7 @@
       <c r="A161">
         <v>160</v>
       </c>
-      <c r="B161" s="15">
+      <c r="B161" s="16">
         <v>14</v>
       </c>
       <c r="C161" s="7" t="s">
@@ -8529,7 +8644,7 @@
       <c r="A162">
         <v>161</v>
       </c>
-      <c r="B162" s="15"/>
+      <c r="B162" s="16"/>
       <c r="C162" s="7" t="s">
         <v>37</v>
       </c>
@@ -8553,7 +8668,7 @@
       <c r="A163">
         <v>162</v>
       </c>
-      <c r="B163" s="15"/>
+      <c r="B163" s="16"/>
       <c r="C163" s="7" t="s">
         <v>38</v>
       </c>
@@ -8577,7 +8692,7 @@
       <c r="A164">
         <v>163</v>
       </c>
-      <c r="B164" s="15"/>
+      <c r="B164" s="16"/>
       <c r="C164" s="7" t="s">
         <v>39</v>
       </c>
@@ -8601,7 +8716,7 @@
       <c r="A165">
         <v>164</v>
       </c>
-      <c r="B165" s="15"/>
+      <c r="B165" s="16"/>
       <c r="C165" s="7" t="s">
         <v>40</v>
       </c>
@@ -8625,7 +8740,7 @@
       <c r="A166">
         <v>165</v>
       </c>
-      <c r="B166" s="15"/>
+      <c r="B166" s="16"/>
       <c r="C166" s="7" t="s">
         <v>41</v>
       </c>
@@ -8649,7 +8764,7 @@
       <c r="A167">
         <v>166</v>
       </c>
-      <c r="B167" s="15"/>
+      <c r="B167" s="16"/>
       <c r="C167" s="7" t="s">
         <v>36</v>
       </c>
@@ -8673,7 +8788,7 @@
       <c r="A168">
         <v>167</v>
       </c>
-      <c r="B168" s="15"/>
+      <c r="B168" s="16"/>
       <c r="C168" s="7" t="s">
         <v>37</v>
       </c>
@@ -8697,7 +8812,7 @@
       <c r="A169">
         <v>168</v>
       </c>
-      <c r="B169" s="15"/>
+      <c r="B169" s="16"/>
       <c r="C169" s="7" t="s">
         <v>38</v>
       </c>
@@ -8721,7 +8836,7 @@
       <c r="A170">
         <v>169</v>
       </c>
-      <c r="B170" s="16">
+      <c r="B170" s="15">
         <v>15</v>
       </c>
       <c r="C170" s="5" t="s">
@@ -8747,7 +8862,7 @@
       <c r="A171">
         <v>170</v>
       </c>
-      <c r="B171" s="16"/>
+      <c r="B171" s="15"/>
       <c r="C171" s="5" t="s">
         <v>40</v>
       </c>
@@ -8771,7 +8886,7 @@
       <c r="A172">
         <v>171</v>
       </c>
-      <c r="B172" s="16"/>
+      <c r="B172" s="15"/>
       <c r="C172" s="5" t="s">
         <v>41</v>
       </c>
@@ -8795,7 +8910,7 @@
       <c r="A173">
         <v>172</v>
       </c>
-      <c r="B173" s="16"/>
+      <c r="B173" s="15"/>
       <c r="C173" s="5" t="s">
         <v>36</v>
       </c>
@@ -8819,7 +8934,7 @@
       <c r="A174">
         <v>173</v>
       </c>
-      <c r="B174" s="16"/>
+      <c r="B174" s="15"/>
       <c r="C174" s="5" t="s">
         <v>37</v>
       </c>
@@ -8843,7 +8958,7 @@
       <c r="A175">
         <v>174</v>
       </c>
-      <c r="B175" s="16"/>
+      <c r="B175" s="15"/>
       <c r="C175" s="5" t="s">
         <v>38</v>
       </c>
@@ -8861,7 +8976,7 @@
       <c r="A176">
         <v>175</v>
       </c>
-      <c r="B176" s="16"/>
+      <c r="B176" s="15"/>
       <c r="C176" s="5" t="s">
         <v>39</v>
       </c>
@@ -8879,7 +8994,7 @@
       <c r="A177">
         <v>176</v>
       </c>
-      <c r="B177" s="16"/>
+      <c r="B177" s="15"/>
       <c r="C177" s="5" t="s">
         <v>40</v>
       </c>
@@ -8897,7 +9012,7 @@
       <c r="A178">
         <v>177</v>
       </c>
-      <c r="B178" s="16"/>
+      <c r="B178" s="15"/>
       <c r="C178" s="5" t="s">
         <v>41</v>
       </c>
@@ -8915,7 +9030,7 @@
       <c r="A179">
         <v>178</v>
       </c>
-      <c r="B179" s="15">
+      <c r="B179" s="16">
         <v>16</v>
       </c>
       <c r="C179" s="7" t="s">
@@ -8941,7 +9056,7 @@
       <c r="A180">
         <v>179</v>
       </c>
-      <c r="B180" s="15"/>
+      <c r="B180" s="16"/>
       <c r="C180" s="7" t="s">
         <v>40</v>
       </c>
@@ -8965,7 +9080,7 @@
       <c r="A181">
         <v>180</v>
       </c>
-      <c r="B181" s="15"/>
+      <c r="B181" s="16"/>
       <c r="C181" s="7" t="s">
         <v>41</v>
       </c>
@@ -8989,7 +9104,7 @@
       <c r="A182">
         <v>181</v>
       </c>
-      <c r="B182" s="15"/>
+      <c r="B182" s="16"/>
       <c r="C182" s="7" t="s">
         <v>36</v>
       </c>
@@ -9013,7 +9128,7 @@
       <c r="A183">
         <v>182</v>
       </c>
-      <c r="B183" s="15"/>
+      <c r="B183" s="16"/>
       <c r="C183" s="7" t="s">
         <v>37</v>
       </c>
@@ -9037,7 +9152,7 @@
       <c r="A184">
         <v>183</v>
       </c>
-      <c r="B184" s="15"/>
+      <c r="B184" s="16"/>
       <c r="C184" s="7" t="s">
         <v>38</v>
       </c>
@@ -9061,7 +9176,7 @@
       <c r="A185">
         <v>184</v>
       </c>
-      <c r="B185" s="15"/>
+      <c r="B185" s="16"/>
       <c r="C185" s="7" t="s">
         <v>39</v>
       </c>
@@ -9085,7 +9200,7 @@
       <c r="A186">
         <v>185</v>
       </c>
-      <c r="B186" s="15"/>
+      <c r="B186" s="16"/>
       <c r="C186" s="7" t="s">
         <v>40</v>
       </c>
@@ -9109,7 +9224,7 @@
       <c r="A187">
         <v>186</v>
       </c>
-      <c r="B187" s="15"/>
+      <c r="B187" s="16"/>
       <c r="C187" s="7" t="s">
         <v>41</v>
       </c>
@@ -9133,7 +9248,7 @@
       <c r="A188">
         <v>187</v>
       </c>
-      <c r="B188" s="15"/>
+      <c r="B188" s="16"/>
       <c r="C188" s="7" t="s">
         <v>36</v>
       </c>
@@ -9157,7 +9272,7 @@
       <c r="A189">
         <v>188</v>
       </c>
-      <c r="B189" s="15"/>
+      <c r="B189" s="16"/>
       <c r="C189" s="7" t="s">
         <v>37</v>
       </c>
@@ -9181,7 +9296,7 @@
       <c r="A190">
         <v>189</v>
       </c>
-      <c r="B190" s="15"/>
+      <c r="B190" s="16"/>
       <c r="C190" s="7" t="s">
         <v>38</v>
       </c>
@@ -9205,7 +9320,7 @@
       <c r="A191">
         <v>190</v>
       </c>
-      <c r="B191" s="16">
+      <c r="B191" s="15">
         <v>17</v>
       </c>
       <c r="C191" s="5" t="s">
@@ -9231,7 +9346,7 @@
       <c r="A192">
         <v>191</v>
       </c>
-      <c r="B192" s="16"/>
+      <c r="B192" s="15"/>
       <c r="C192" s="5" t="s">
         <v>37</v>
       </c>
@@ -9255,7 +9370,7 @@
       <c r="A193">
         <v>192</v>
       </c>
-      <c r="B193" s="16"/>
+      <c r="B193" s="15"/>
       <c r="C193" s="5" t="s">
         <v>38</v>
       </c>
@@ -9279,7 +9394,7 @@
       <c r="A194">
         <v>193</v>
       </c>
-      <c r="B194" s="16"/>
+      <c r="B194" s="15"/>
       <c r="C194" s="5" t="s">
         <v>39</v>
       </c>
@@ -9303,7 +9418,7 @@
       <c r="A195">
         <v>194</v>
       </c>
-      <c r="B195" s="16"/>
+      <c r="B195" s="15"/>
       <c r="C195" s="5" t="s">
         <v>40</v>
       </c>
@@ -9327,7 +9442,7 @@
       <c r="A196">
         <v>195</v>
       </c>
-      <c r="B196" s="16"/>
+      <c r="B196" s="15"/>
       <c r="C196" s="5" t="s">
         <v>41</v>
       </c>
@@ -9351,7 +9466,7 @@
       <c r="A197">
         <v>196</v>
       </c>
-      <c r="B197" s="16"/>
+      <c r="B197" s="15"/>
       <c r="C197" s="5" t="s">
         <v>36</v>
       </c>
@@ -9375,7 +9490,7 @@
       <c r="A198">
         <v>197</v>
       </c>
-      <c r="B198" s="16"/>
+      <c r="B198" s="15"/>
       <c r="C198" s="5" t="s">
         <v>37</v>
       </c>
@@ -9399,7 +9514,7 @@
       <c r="A199">
         <v>198</v>
       </c>
-      <c r="B199" s="16"/>
+      <c r="B199" s="15"/>
       <c r="C199" s="5" t="s">
         <v>38</v>
       </c>
@@ -9423,7 +9538,7 @@
       <c r="A200">
         <v>199</v>
       </c>
-      <c r="B200" s="15">
+      <c r="B200" s="16">
         <v>18</v>
       </c>
       <c r="C200" s="7" t="s">
@@ -9449,7 +9564,7 @@
       <c r="A201">
         <v>200</v>
       </c>
-      <c r="B201" s="15"/>
+      <c r="B201" s="16"/>
       <c r="C201" s="7" t="s">
         <v>40</v>
       </c>
@@ -9473,7 +9588,7 @@
       <c r="A202">
         <v>201</v>
       </c>
-      <c r="B202" s="15"/>
+      <c r="B202" s="16"/>
       <c r="C202" s="7" t="s">
         <v>41</v>
       </c>
@@ -9497,7 +9612,7 @@
       <c r="A203">
         <v>202</v>
       </c>
-      <c r="B203" s="15"/>
+      <c r="B203" s="16"/>
       <c r="C203" s="7" t="s">
         <v>36</v>
       </c>
@@ -9521,7 +9636,7 @@
       <c r="A204">
         <v>203</v>
       </c>
-      <c r="B204" s="15"/>
+      <c r="B204" s="16"/>
       <c r="C204" s="7" t="s">
         <v>37</v>
       </c>
@@ -9545,7 +9660,7 @@
       <c r="A205">
         <v>204</v>
       </c>
-      <c r="B205" s="15"/>
+      <c r="B205" s="16"/>
       <c r="C205" s="7" t="s">
         <v>38</v>
       </c>
@@ -9569,7 +9684,7 @@
       <c r="A206">
         <v>205</v>
       </c>
-      <c r="B206" s="15"/>
+      <c r="B206" s="16"/>
       <c r="C206" s="7" t="s">
         <v>39</v>
       </c>
@@ -9593,7 +9708,7 @@
       <c r="A207">
         <v>206</v>
       </c>
-      <c r="B207" s="15"/>
+      <c r="B207" s="16"/>
       <c r="C207" s="7" t="s">
         <v>40</v>
       </c>
@@ -9617,7 +9732,7 @@
       <c r="A208">
         <v>207</v>
       </c>
-      <c r="B208" s="15"/>
+      <c r="B208" s="16"/>
       <c r="C208" s="7" t="s">
         <v>41</v>
       </c>
@@ -9641,7 +9756,7 @@
       <c r="A209">
         <v>208</v>
       </c>
-      <c r="B209" s="16">
+      <c r="B209" s="15">
         <v>19</v>
       </c>
       <c r="C209" s="5" t="s">
@@ -9661,7 +9776,7 @@
       <c r="A210">
         <v>209</v>
       </c>
-      <c r="B210" s="16"/>
+      <c r="B210" s="15"/>
       <c r="C210" s="5" t="s">
         <v>37</v>
       </c>
@@ -9679,7 +9794,7 @@
       <c r="A211">
         <v>210</v>
       </c>
-      <c r="B211" s="16"/>
+      <c r="B211" s="15"/>
       <c r="C211" s="5" t="s">
         <v>38</v>
       </c>
@@ -9697,7 +9812,7 @@
       <c r="A212">
         <v>211</v>
       </c>
-      <c r="B212" s="16"/>
+      <c r="B212" s="15"/>
       <c r="C212" s="5" t="s">
         <v>39</v>
       </c>
@@ -9721,7 +9836,7 @@
       <c r="A213">
         <v>212</v>
       </c>
-      <c r="B213" s="16"/>
+      <c r="B213" s="15"/>
       <c r="C213" s="5" t="s">
         <v>40</v>
       </c>
@@ -9745,7 +9860,7 @@
       <c r="A214">
         <v>213</v>
       </c>
-      <c r="B214" s="16"/>
+      <c r="B214" s="15"/>
       <c r="C214" s="5" t="s">
         <v>41</v>
       </c>
@@ -9769,7 +9884,7 @@
       <c r="A215">
         <v>214</v>
       </c>
-      <c r="B215" s="16"/>
+      <c r="B215" s="15"/>
       <c r="C215" s="5" t="s">
         <v>42</v>
       </c>
@@ -9793,7 +9908,7 @@
       <c r="A216">
         <v>215</v>
       </c>
-      <c r="B216" s="16"/>
+      <c r="B216" s="15"/>
       <c r="C216" s="5" t="s">
         <v>43</v>
       </c>
@@ -9817,7 +9932,7 @@
       <c r="A217">
         <v>216</v>
       </c>
-      <c r="B217" s="16"/>
+      <c r="B217" s="15"/>
       <c r="C217" s="5" t="s">
         <v>44</v>
       </c>
@@ -9841,7 +9956,7 @@
       <c r="A218">
         <v>217</v>
       </c>
-      <c r="B218" s="16"/>
+      <c r="B218" s="15"/>
       <c r="C218" s="5" t="s">
         <v>45</v>
       </c>
@@ -9865,7 +9980,7 @@
       <c r="A219">
         <v>218</v>
       </c>
-      <c r="B219" s="16"/>
+      <c r="B219" s="15"/>
       <c r="C219" s="5" t="s">
         <v>46</v>
       </c>
@@ -9889,7 +10004,7 @@
       <c r="A220">
         <v>219</v>
       </c>
-      <c r="B220" s="16"/>
+      <c r="B220" s="15"/>
       <c r="C220" s="5" t="s">
         <v>47</v>
       </c>
@@ -9913,7 +10028,7 @@
       <c r="A221">
         <v>220</v>
       </c>
-      <c r="B221" s="16"/>
+      <c r="B221" s="15"/>
       <c r="C221" s="5" t="s">
         <v>48</v>
       </c>
@@ -9937,7 +10052,7 @@
       <c r="A222">
         <v>221</v>
       </c>
-      <c r="B222" s="16"/>
+      <c r="B222" s="15"/>
       <c r="C222" s="5" t="s">
         <v>36</v>
       </c>
@@ -9961,7 +10076,7 @@
       <c r="A223">
         <v>222</v>
       </c>
-      <c r="B223" s="16"/>
+      <c r="B223" s="15"/>
       <c r="C223" s="5" t="s">
         <v>37</v>
       </c>
@@ -9985,7 +10100,7 @@
       <c r="A224">
         <v>223</v>
       </c>
-      <c r="B224" s="16"/>
+      <c r="B224" s="15"/>
       <c r="C224" s="5" t="s">
         <v>38</v>
       </c>
@@ -10009,7 +10124,7 @@
       <c r="A225">
         <v>224</v>
       </c>
-      <c r="B225" s="16"/>
+      <c r="B225" s="15"/>
       <c r="C225" s="5" t="s">
         <v>49</v>
       </c>
@@ -10033,7 +10148,7 @@
       <c r="A226">
         <v>225</v>
       </c>
-      <c r="B226" s="16"/>
+      <c r="B226" s="15"/>
       <c r="C226" s="5" t="s">
         <v>50</v>
       </c>
@@ -10057,7 +10172,7 @@
       <c r="A227">
         <v>226</v>
       </c>
-      <c r="B227" s="16"/>
+      <c r="B227" s="15"/>
       <c r="C227" s="5" t="s">
         <v>51</v>
       </c>
@@ -10081,7 +10196,7 @@
       <c r="A228">
         <v>227</v>
       </c>
-      <c r="B228" s="16"/>
+      <c r="B228" s="15"/>
       <c r="C228" s="5" t="s">
         <v>52</v>
       </c>
@@ -10102,209 +10217,930 @@
       </c>
     </row>
     <row r="229" spans="1:8">
-      <c r="A229">
+      <c r="A229" s="17">
         <v>228</v>
       </c>
-      <c r="B229" s="18">
+      <c r="B229" s="19">
         <v>20</v>
       </c>
-      <c r="C229" s="19" t="s">
+      <c r="C229" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="D229" s="18">
+        <v>46311</v>
+      </c>
+      <c r="E229" s="17">
+        <v>0.63900000000000001</v>
+      </c>
+      <c r="F229" s="17">
+        <v>0.52</v>
+      </c>
+      <c r="G229" s="17">
+        <v>9.7100000000000009</v>
+      </c>
+      <c r="H229" s="20" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="230" spans="1:8">
+      <c r="A230" s="17">
+        <v>229</v>
+      </c>
+      <c r="B230" s="21"/>
+      <c r="C230" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="D230" s="18">
+        <v>46311</v>
+      </c>
+      <c r="E230" s="17">
+        <v>0.61799999999999999</v>
+      </c>
+      <c r="F230" s="17">
+        <v>0.52</v>
+      </c>
+      <c r="G230" s="17">
+        <v>9.0399999999999991</v>
+      </c>
+      <c r="H230" s="20" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="231" spans="1:8">
+      <c r="A231" s="17">
+        <v>230</v>
+      </c>
+      <c r="B231" s="21"/>
+      <c r="C231" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D231" s="18">
+        <v>46311</v>
+      </c>
+      <c r="E231" s="17">
+        <v>0.67700000000000005</v>
+      </c>
+      <c r="F231" s="17">
+        <v>0.53</v>
+      </c>
+      <c r="G231" s="17">
+        <v>9.44</v>
+      </c>
+      <c r="H231" s="20" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="232" spans="1:8">
+      <c r="A232" s="17">
+        <v>231</v>
+      </c>
+      <c r="B232" s="21"/>
+      <c r="C232" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="D232" s="18">
+        <v>46311</v>
+      </c>
+      <c r="E232" s="17">
+        <v>0.63300000000000001</v>
+      </c>
+      <c r="F232" s="17">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G232" s="17">
+        <v>9.4499999999999993</v>
+      </c>
+      <c r="H232" s="20" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="233" spans="1:8">
+      <c r="A233" s="17">
+        <v>232</v>
+      </c>
+      <c r="B233" s="21"/>
+      <c r="C233" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="D233" s="18">
+        <v>46311</v>
+      </c>
+      <c r="E233" s="17">
+        <v>0.60099999999999998</v>
+      </c>
+      <c r="F233" s="17">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G233" s="17">
+        <v>9.57</v>
+      </c>
+      <c r="H233" s="20" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="234" spans="1:8">
+      <c r="A234" s="17">
+        <v>233</v>
+      </c>
+      <c r="B234" s="21"/>
+      <c r="C234" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="D234" s="18">
+        <v>46311</v>
+      </c>
+      <c r="E234" s="17">
+        <v>0.60899999999999999</v>
+      </c>
+      <c r="F234" s="17">
+        <v>0.61</v>
+      </c>
+      <c r="G234" s="17">
+        <v>9.4</v>
+      </c>
+      <c r="H234" s="20" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="235" spans="1:8">
+      <c r="A235" s="17">
+        <v>234</v>
+      </c>
+      <c r="B235" s="21"/>
+      <c r="C235" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="D235" s="18">
+        <v>46311</v>
+      </c>
+      <c r="E235" s="17">
+        <v>0.64900000000000002</v>
+      </c>
+      <c r="F235" s="17">
+        <v>0.51</v>
+      </c>
+      <c r="G235" s="17">
+        <v>9.1999999999999993</v>
+      </c>
+      <c r="H235" s="20" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="236" spans="1:8">
+      <c r="A236" s="17">
+        <v>235</v>
+      </c>
+      <c r="B236" s="21"/>
+      <c r="C236" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="D236" s="18">
+        <v>46311</v>
+      </c>
+      <c r="E236" s="17">
+        <v>0.66500000000000004</v>
+      </c>
+      <c r="F236" s="17">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G236" s="17">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="H236" s="20" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="237" spans="1:8">
+      <c r="A237" s="17">
+        <v>236</v>
+      </c>
+      <c r="B237" s="21"/>
+      <c r="C237" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="D237" s="18">
+        <v>46311</v>
+      </c>
+      <c r="E237" s="17">
+        <v>0.64</v>
+      </c>
+      <c r="F237" s="17">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G237" s="17">
+        <v>9.2100000000000009</v>
+      </c>
+      <c r="H237" s="22" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="238" spans="1:8">
+      <c r="A238" s="17">
+        <v>237</v>
+      </c>
+      <c r="B238" s="21"/>
+      <c r="C238" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="D238" s="18">
+        <v>46311</v>
+      </c>
+      <c r="E238" s="17">
+        <v>0.64500000000000002</v>
+      </c>
+      <c r="F238" s="17">
+        <v>0.51</v>
+      </c>
+      <c r="G238" s="17">
+        <v>9.18</v>
+      </c>
+      <c r="H238" s="22" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="239" spans="1:8">
+      <c r="A239" s="17">
+        <v>238</v>
+      </c>
+      <c r="B239" s="21"/>
+      <c r="C239" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="D229" s="17">
+      <c r="D239" s="18">
         <v>46312</v>
       </c>
-      <c r="E229" s="19">
+      <c r="E239" s="17">
         <v>0.63200000000000001</v>
       </c>
-      <c r="F229" s="19">
+      <c r="F239" s="17">
         <v>0.57999999999999996</v>
       </c>
-      <c r="G229" s="19">
+      <c r="G239" s="17">
         <v>8.07</v>
       </c>
-      <c r="H229" s="20" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="230" spans="1:8">
-      <c r="A230">
-        <v>229</v>
-      </c>
-      <c r="B230" s="18"/>
-      <c r="C230" s="19" t="s">
+      <c r="H239" s="22" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="240" spans="1:8">
+      <c r="A240" s="17">
+        <v>239</v>
+      </c>
+      <c r="B240" s="21"/>
+      <c r="C240" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="D230" s="17">
+      <c r="D240" s="18">
         <v>46312</v>
       </c>
-      <c r="E230" s="19">
+      <c r="E240" s="17">
         <v>0.68600000000000005</v>
       </c>
-      <c r="F230" s="19">
+      <c r="F240" s="17">
         <v>0.56000000000000005</v>
       </c>
-      <c r="G230" s="19">
+      <c r="G240" s="17">
         <v>8.31</v>
       </c>
-      <c r="H230" s="20" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="231" spans="1:8">
-      <c r="A231">
-        <v>230</v>
-      </c>
-      <c r="B231" s="18"/>
-      <c r="C231" s="19" t="s">
+      <c r="H240" s="22" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="241" spans="1:8">
+      <c r="A241" s="17">
+        <v>240</v>
+      </c>
+      <c r="B241" s="21"/>
+      <c r="C241" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="D231" s="17">
+      <c r="D241" s="18">
         <v>46312</v>
       </c>
-      <c r="E231" s="19">
+      <c r="E241" s="17">
         <v>0.69</v>
       </c>
-      <c r="F231" s="19">
+      <c r="F241" s="17">
         <v>0.52</v>
       </c>
-      <c r="G231" s="19">
+      <c r="G241" s="17">
         <v>8.7899999999999991</v>
       </c>
-      <c r="H231" s="20" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="232" spans="1:8">
-      <c r="A232">
-        <v>231</v>
-      </c>
-      <c r="B232" s="18"/>
-      <c r="C232" s="19" t="s">
+      <c r="H241" s="22" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="242" spans="1:8">
+      <c r="A242" s="17">
+        <v>241</v>
+      </c>
+      <c r="B242" s="21"/>
+      <c r="C242" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="D232" s="17">
+      <c r="D242" s="18">
         <v>46312</v>
       </c>
-      <c r="E232" s="19">
+      <c r="E242" s="17">
         <v>0.75900000000000001</v>
       </c>
-      <c r="F232" s="19">
+      <c r="F242" s="17">
         <v>0.53</v>
       </c>
-      <c r="G232" s="19">
+      <c r="G242" s="17">
         <v>8.43</v>
       </c>
-      <c r="H232" s="20" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="233" spans="1:8">
-      <c r="A233">
-        <v>232</v>
-      </c>
-      <c r="B233" s="18"/>
-      <c r="C233" s="19" t="s">
+      <c r="H242" s="22" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="243" spans="1:8">
+      <c r="A243" s="17">
+        <v>242</v>
+      </c>
+      <c r="B243" s="21"/>
+      <c r="C243" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="D233" s="17">
+      <c r="D243" s="18">
         <v>46312</v>
       </c>
-      <c r="E233" s="19">
+      <c r="E243" s="17">
         <v>0.746</v>
       </c>
-      <c r="F233" s="19">
+      <c r="F243" s="17">
         <v>0.55000000000000004</v>
       </c>
-      <c r="G233" s="19">
+      <c r="G243" s="17">
         <v>8.5500000000000007</v>
       </c>
-      <c r="H233" s="20" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="234" spans="1:8">
-      <c r="A234">
-        <v>233</v>
-      </c>
-      <c r="B234" s="18"/>
-      <c r="C234" s="19" t="s">
+      <c r="H243" s="22"/>
+    </row>
+    <row r="244" spans="1:8">
+      <c r="A244" s="17">
+        <v>243</v>
+      </c>
+      <c r="B244" s="21"/>
+      <c r="C244" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="D234" s="17">
+      <c r="D244" s="18">
         <v>46312</v>
       </c>
-      <c r="E234" s="19">
+      <c r="E244" s="17">
         <v>0.73299999999999998</v>
       </c>
-      <c r="F234" s="19">
+      <c r="F244" s="17">
         <v>0.55000000000000004</v>
       </c>
-      <c r="G234" s="19">
+      <c r="G244" s="17">
         <v>8.49</v>
       </c>
-      <c r="H234" s="20" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="235" spans="1:8">
-      <c r="A235">
-        <v>234</v>
-      </c>
-      <c r="B235" s="18"/>
-      <c r="C235" s="19" t="s">
+      <c r="H244" s="22"/>
+    </row>
+    <row r="245" spans="1:8">
+      <c r="A245" s="17">
+        <v>244</v>
+      </c>
+      <c r="B245" s="21"/>
+      <c r="C245" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="D235" s="17">
+      <c r="D245" s="18">
         <v>46312</v>
       </c>
-      <c r="E235" s="19">
+      <c r="E245" s="17">
         <v>0.72499999999999998</v>
       </c>
-      <c r="F235" s="19">
+      <c r="F245" s="17">
         <v>0.53</v>
       </c>
-      <c r="G235" s="19">
+      <c r="G245" s="17">
         <v>8.14</v>
       </c>
-      <c r="H235" s="20" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="236" spans="1:8">
-      <c r="A236">
-        <v>235</v>
-      </c>
-      <c r="B236" s="18"/>
-      <c r="C236" s="19" t="s">
+      <c r="H245" s="22"/>
+    </row>
+    <row r="246" spans="1:8">
+      <c r="A246" s="17">
+        <v>245</v>
+      </c>
+      <c r="B246" s="23"/>
+      <c r="C246" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="D236" s="17">
+      <c r="D246" s="18">
         <v>46312</v>
       </c>
-      <c r="E236" s="19">
+      <c r="E246" s="17">
         <v>0.73</v>
       </c>
-      <c r="F236" s="19">
+      <c r="F246" s="17">
         <v>0.57999999999999996</v>
       </c>
-      <c r="G236" s="19">
+      <c r="G246" s="17">
         <v>8.57</v>
       </c>
-      <c r="H236" s="20" t="s">
-        <v>29</v>
-      </c>
+      <c r="H246" s="22"/>
+    </row>
+    <row r="247" spans="1:8">
+      <c r="A247" s="24">
+        <v>246</v>
+      </c>
+      <c r="B247" s="25">
+        <v>21</v>
+      </c>
+      <c r="C247" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="D247" s="26">
+        <v>46313</v>
+      </c>
+      <c r="E247" s="24">
+        <v>0.51100000000000001</v>
+      </c>
+      <c r="F247" s="24">
+        <v>0.61</v>
+      </c>
+      <c r="G247" s="24">
+        <v>10.76</v>
+      </c>
+    </row>
+    <row r="248" spans="1:8">
+      <c r="A248" s="24">
+        <v>247</v>
+      </c>
+      <c r="B248" s="25"/>
+      <c r="C248" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="D248" s="26">
+        <v>46313</v>
+      </c>
+      <c r="E248" s="24">
+        <v>0.46899999999999997</v>
+      </c>
+      <c r="F248" s="24">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="G248" s="24">
+        <v>11.27</v>
+      </c>
+    </row>
+    <row r="249" spans="1:8">
+      <c r="A249" s="24">
+        <v>248</v>
+      </c>
+      <c r="B249" s="25"/>
+      <c r="C249" s="24" t="s">
+        <v>38</v>
+      </c>
+      <c r="D249" s="26">
+        <v>46313</v>
+      </c>
+      <c r="E249" s="24">
+        <v>0.45</v>
+      </c>
+      <c r="F249" s="24">
+        <v>0.59</v>
+      </c>
+      <c r="G249" s="24">
+        <v>10.95</v>
+      </c>
+    </row>
+    <row r="250" spans="1:8">
+      <c r="A250" s="24">
+        <v>249</v>
+      </c>
+      <c r="B250" s="25"/>
+      <c r="C250" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="D250" s="26">
+        <v>46313</v>
+      </c>
+      <c r="E250" s="24">
+        <v>0.50700000000000001</v>
+      </c>
+      <c r="F250" s="24">
+        <v>0.5</v>
+      </c>
+      <c r="G250" s="24">
+        <v>10.75</v>
+      </c>
+    </row>
+    <row r="251" spans="1:8">
+      <c r="A251" s="24">
+        <v>250</v>
+      </c>
+      <c r="B251" s="25"/>
+      <c r="C251" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="D251" s="26">
+        <v>46313</v>
+      </c>
+      <c r="E251" s="24">
+        <v>0.49399999999999999</v>
+      </c>
+      <c r="F251" s="24">
+        <v>0.53</v>
+      </c>
+      <c r="G251" s="24">
+        <v>10.36</v>
+      </c>
+    </row>
+    <row r="252" spans="1:8">
+      <c r="A252" s="24">
+        <v>251</v>
+      </c>
+      <c r="B252" s="25"/>
+      <c r="C252" s="24" t="s">
+        <v>51</v>
+      </c>
+      <c r="D252" s="26">
+        <v>46313</v>
+      </c>
+      <c r="E252" s="24">
+        <v>0.56599999999999995</v>
+      </c>
+      <c r="F252" s="24">
+        <v>0.47</v>
+      </c>
+      <c r="G252" s="24">
+        <v>10.43</v>
+      </c>
+    </row>
+    <row r="253" spans="1:8">
+      <c r="A253" s="24">
+        <v>252</v>
+      </c>
+      <c r="B253" s="25"/>
+      <c r="C253" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="D253" s="26">
+        <v>46313</v>
+      </c>
+      <c r="E253" s="24">
+        <v>0.36299999999999999</v>
+      </c>
+      <c r="F253" s="24">
+        <v>0.17599999999999999</v>
+      </c>
+      <c r="G253" s="24">
+        <v>8.0760000000000005</v>
+      </c>
+    </row>
+    <row r="254" spans="1:8">
+      <c r="A254" s="24">
+        <v>253</v>
+      </c>
+      <c r="B254" s="25"/>
+      <c r="C254" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="D254" s="26">
+        <v>46313</v>
+      </c>
+      <c r="E254" s="24">
+        <v>0.317</v>
+      </c>
+      <c r="F254" s="24">
+        <v>0.27400000000000002</v>
+      </c>
+      <c r="G254" s="24">
+        <v>8.1120000000000001</v>
+      </c>
+    </row>
+    <row r="255" spans="1:8">
+      <c r="A255" s="24">
+        <v>254</v>
+      </c>
+      <c r="B255" s="25"/>
+      <c r="C255" s="24" t="s">
+        <v>38</v>
+      </c>
+      <c r="D255" s="26">
+        <v>46313</v>
+      </c>
+      <c r="E255" s="24">
+        <v>0.36399999999999999</v>
+      </c>
+      <c r="F255" s="24">
+        <v>0.16500000000000001</v>
+      </c>
+      <c r="G255" s="24">
+        <v>8.5830000000000002</v>
+      </c>
+    </row>
+    <row r="256" spans="1:8">
+      <c r="A256" s="24">
+        <v>255</v>
+      </c>
+      <c r="B256" s="25"/>
+      <c r="C256" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="D256" s="26">
+        <v>46313</v>
+      </c>
+      <c r="E256" s="24">
+        <v>0.26100000000000001</v>
+      </c>
+      <c r="F256" s="24">
+        <v>0.17</v>
+      </c>
+      <c r="G256" s="24">
+        <v>6.79</v>
+      </c>
+    </row>
+    <row r="257" spans="1:7">
+      <c r="A257" s="24">
+        <v>256</v>
+      </c>
+      <c r="B257" s="25"/>
+      <c r="C257" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="D257" s="26">
+        <v>46313</v>
+      </c>
+      <c r="E257" s="24">
+        <v>0.30599999999999999</v>
+      </c>
+      <c r="F257" s="24">
+        <v>0.3</v>
+      </c>
+      <c r="G257" s="24">
+        <v>5.55</v>
+      </c>
+    </row>
+    <row r="258" spans="1:7">
+      <c r="A258" s="24">
+        <v>257</v>
+      </c>
+      <c r="B258" s="25"/>
+      <c r="C258" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="D258" s="26">
+        <v>46313</v>
+      </c>
+      <c r="E258" s="24">
+        <v>0.379</v>
+      </c>
+      <c r="F258" s="24">
+        <v>0.20499999999999999</v>
+      </c>
+      <c r="G258" s="24">
+        <v>9.859</v>
+      </c>
+    </row>
+    <row r="259" spans="1:7">
+      <c r="A259" s="24">
+        <v>258</v>
+      </c>
+      <c r="B259" s="25"/>
+      <c r="C259" s="24" t="s">
+        <v>40</v>
+      </c>
+      <c r="D259" s="26">
+        <v>46313</v>
+      </c>
+      <c r="E259" s="24">
+        <v>0.35199999999999998</v>
+      </c>
+      <c r="F259" s="24">
+        <v>0.36699999999999999</v>
+      </c>
+      <c r="G259" s="24">
+        <v>10.090999999999999</v>
+      </c>
+    </row>
+    <row r="260" spans="1:7">
+      <c r="A260" s="24">
+        <v>259</v>
+      </c>
+      <c r="B260" s="25"/>
+      <c r="C260" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="D260" s="26">
+        <v>46313</v>
+      </c>
+      <c r="E260" s="24">
+        <v>0.50600000000000001</v>
+      </c>
+      <c r="F260" s="24">
+        <v>0.21199999999999999</v>
+      </c>
+      <c r="G260" s="24">
+        <v>9.9169999999999998</v>
+      </c>
+    </row>
+    <row r="261" spans="1:7">
+      <c r="A261" s="24">
+        <v>260</v>
+      </c>
+      <c r="B261" s="25"/>
+      <c r="C261" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="D261" s="26">
+        <v>46313</v>
+      </c>
+      <c r="E261" s="24">
+        <v>0.435</v>
+      </c>
+      <c r="F261" s="24">
+        <v>0.27600000000000002</v>
+      </c>
+      <c r="G261" s="24">
+        <v>9.5419999999999998</v>
+      </c>
+    </row>
+    <row r="262" spans="1:7">
+      <c r="A262" s="24">
+        <v>261</v>
+      </c>
+      <c r="B262" s="25"/>
+      <c r="C262" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="D262" s="26">
+        <v>46313</v>
+      </c>
+      <c r="E262" s="24">
+        <v>0.46300000000000002</v>
+      </c>
+      <c r="F262" s="24">
+        <v>0.30099999999999999</v>
+      </c>
+      <c r="G262" s="24">
+        <v>9.6780000000000008</v>
+      </c>
+    </row>
+    <row r="263" spans="1:7">
+      <c r="A263" s="24">
+        <v>262</v>
+      </c>
+      <c r="B263" s="25"/>
+      <c r="C263" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="D263" s="26">
+        <v>46313</v>
+      </c>
+      <c r="E263" s="24">
+        <v>0.33</v>
+      </c>
+      <c r="F263" s="24">
+        <v>0.15</v>
+      </c>
+      <c r="G263" s="24">
+        <v>7.61</v>
+      </c>
+    </row>
+    <row r="264" spans="1:7">
+      <c r="A264" s="24">
+        <v>263</v>
+      </c>
+      <c r="B264" s="25"/>
+      <c r="C264" s="24" t="s">
+        <v>40</v>
+      </c>
+      <c r="D264" s="26">
+        <v>46313</v>
+      </c>
+      <c r="E264" s="24">
+        <v>0.311</v>
+      </c>
+      <c r="F264" s="24">
+        <v>0.36</v>
+      </c>
+      <c r="G264" s="24">
+        <v>9.0399999999999991</v>
+      </c>
+    </row>
+    <row r="265" spans="1:7">
+      <c r="A265" s="24">
+        <v>264</v>
+      </c>
+      <c r="B265" s="25"/>
+      <c r="C265" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="D265" s="26">
+        <v>46314</v>
+      </c>
+      <c r="E265" s="24">
+        <v>0.443</v>
+      </c>
+      <c r="F265" s="24">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="G265" s="24">
+        <v>12.67</v>
+      </c>
+    </row>
+    <row r="266" spans="1:7">
+      <c r="A266" s="24">
+        <v>265</v>
+      </c>
+      <c r="B266" s="25"/>
+      <c r="C266" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="D266" s="26">
+        <v>46314</v>
+      </c>
+      <c r="E266" s="24">
+        <v>0.45600000000000002</v>
+      </c>
+      <c r="F266" s="24">
+        <v>0.68</v>
+      </c>
+      <c r="G266" s="24">
+        <v>12.38</v>
+      </c>
+    </row>
+    <row r="267" spans="1:7">
+      <c r="A267" s="24">
+        <v>266</v>
+      </c>
+      <c r="B267" s="25"/>
+      <c r="C267" s="24" t="s">
+        <v>38</v>
+      </c>
+      <c r="D267" s="26">
+        <v>46314</v>
+      </c>
+      <c r="E267" s="24">
+        <v>0.47399999999999998</v>
+      </c>
+      <c r="F267" s="24">
+        <v>0.6</v>
+      </c>
+      <c r="G267" s="24">
+        <v>13.18</v>
+      </c>
+    </row>
+    <row r="268" spans="1:7">
+      <c r="A268" s="24">
+        <v>267</v>
+      </c>
+      <c r="B268" s="25"/>
+      <c r="C268" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="D268" s="26">
+        <v>46314</v>
+      </c>
+      <c r="E268" s="24">
+        <v>0.46300000000000002</v>
+      </c>
+      <c r="F268" s="24">
+        <v>0.17</v>
+      </c>
+      <c r="G268" s="24">
+        <v>10.220000000000001</v>
+      </c>
+    </row>
+    <row r="269" spans="1:7">
+      <c r="A269" s="24">
+        <v>268</v>
+      </c>
+      <c r="B269" s="25"/>
+      <c r="C269" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="D269" s="26">
+        <v>46314</v>
+      </c>
+      <c r="E269" s="24">
+        <v>0.38700000000000001</v>
+      </c>
+      <c r="F269" s="24">
+        <v>0.32</v>
+      </c>
+      <c r="G269" s="24">
+        <v>9.85</v>
+      </c>
+    </row>
+    <row r="270" spans="1:7">
+      <c r="A270" s="24">
+        <v>269</v>
+      </c>
+      <c r="B270" s="25"/>
+      <c r="C270" s="24"/>
+      <c r="D270" s="26"/>
+      <c r="E270" s="24"/>
+      <c r="F270" s="24"/>
+      <c r="G270" s="24"/>
     </row>
   </sheetData>
-  <mergeCells count="20">
-    <mergeCell ref="B229:B236"/>
-    <mergeCell ref="B209:B228"/>
-    <mergeCell ref="B146:B160"/>
-    <mergeCell ref="B161:B169"/>
-    <mergeCell ref="B170:B178"/>
-    <mergeCell ref="B179:B190"/>
-    <mergeCell ref="B191:B199"/>
-    <mergeCell ref="B200:B208"/>
+  <mergeCells count="21">
+    <mergeCell ref="B247:B270"/>
     <mergeCell ref="B128:B145"/>
     <mergeCell ref="B2:B13"/>
     <mergeCell ref="B14:B22"/>
@@ -10317,7 +11153,16 @@
     <mergeCell ref="B86:B97"/>
     <mergeCell ref="B98:B118"/>
     <mergeCell ref="B119:B127"/>
+    <mergeCell ref="B209:B228"/>
+    <mergeCell ref="B146:B160"/>
+    <mergeCell ref="B161:B169"/>
+    <mergeCell ref="B170:B178"/>
+    <mergeCell ref="B179:B190"/>
+    <mergeCell ref="B191:B199"/>
+    <mergeCell ref="B200:B208"/>
+    <mergeCell ref="B229:B246"/>
   </mergeCells>
+  <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>